<commit_message>
chore: update sec 62 sem1,3,5
</commit_message>
<xml_diff>
--- a/raw/time_tables/B.Tech 62 (btech-62)/1/1.xlsx
+++ b/raw/time_tables/B.Tech 62 (btech-62)/1/1.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -65,16 +65,6 @@
       <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <color rgb="00FF0000"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Times New Roman"/>
-      <color rgb="00FF0000"/>
-      <sz val="11"/>
-    </font>
-    <font>
       <name val="Times New Roman"/>
       <b val="1"/>
       <color rgb="00FF0000"/>
@@ -83,6 +73,11 @@
     <font>
       <name val="Times New Roman"/>
       <b val="1"/>
+      <color rgb="00FF0000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <color rgb="00FF0000"/>
       <sz val="11"/>
     </font>
@@ -104,12 +99,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -321,7 +316,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
@@ -373,11 +368,7 @@
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -386,10 +377,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="center" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -403,16 +390,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -439,11 +422,11 @@
       <alignment horizontal="general" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -451,7 +434,7 @@
       <alignment horizontal="general" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -459,11 +442,7 @@
       <alignment horizontal="general" vertical="bottom" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -1331,7 +1310,7 @@
       </c>
       <c r="H5" s="10" t="inlineStr">
         <is>
-          <t>LA15,A16(CI111)-FF2/ROH</t>
+          <t>LA15,A16(CI111)-FF2/RJM</t>
         </is>
       </c>
       <c r="I5" s="10" t="inlineStr">
@@ -1594,7 +1573,11 @@
           <t>LB11,B12(CI111)-CR425/SHY</t>
         </is>
       </c>
-      <c r="I10" s="14" t="inlineStr"/>
+      <c r="I10" s="14" t="inlineStr">
+        <is>
+          <t>LB1,B2(CI111)-G7/TNV</t>
+        </is>
+      </c>
       <c r="J10" s="5" t="inlineStr"/>
       <c r="K10" s="1" t="inlineStr"/>
       <c r="L10" s="1" t="inlineStr"/>
@@ -1625,7 +1608,7 @@
       <c r="E11" s="11" t="n"/>
       <c r="F11" s="10" t="inlineStr">
         <is>
-          <t>LG5,G6(CI111)-G7/SMS</t>
+          <t>LG5,G6(CI111)-G7/PAG</t>
         </is>
       </c>
       <c r="G11" s="10" t="inlineStr">
@@ -1638,7 +1621,7 @@
           <t>LG3,G4(CI111)-CR501/SHO</t>
         </is>
       </c>
-      <c r="I11" s="15" t="inlineStr"/>
+      <c r="I11" s="1" t="inlineStr"/>
       <c r="J11" s="5" t="inlineStr"/>
       <c r="K11" s="1" t="inlineStr"/>
       <c r="L11" s="1" t="inlineStr"/>
@@ -1785,7 +1768,7 @@
       <c r="A15" s="11" t="n"/>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>TA4(CI111)-TS8PSO</t>
+          <t>TA4(CI111)-TS8/AYS</t>
         </is>
       </c>
       <c r="C15" s="10" t="inlineStr">
@@ -2070,7 +2053,7 @@
       <c r="F21" s="10" t="inlineStr"/>
       <c r="G21" s="10" t="inlineStr">
         <is>
-          <t>TD2(CI111)-TR307/PKU</t>
+          <t>TD2(CI111)-TR307/SRG</t>
         </is>
       </c>
       <c r="H21" s="10" t="inlineStr">
@@ -2216,9 +2199,9 @@
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="11" t="n"/>
       <c r="B25" s="12" t="inlineStr"/>
-      <c r="C25" s="16" t="inlineStr">
-        <is>
-          <t>PG5(CS111)-AVR,DSI/CL01</t>
+      <c r="C25" s="15" t="inlineStr">
+        <is>
+          <t>PG4,G5(CS111)-AVR,DSI,AW/CL01,02</t>
         </is>
       </c>
       <c r="D25" s="4" t="n"/>
@@ -2256,11 +2239,7 @@
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="11" t="n"/>
       <c r="B26" s="12" t="inlineStr"/>
-      <c r="C26" s="16" t="inlineStr">
-        <is>
-          <t>PG4(CS111)-AW,SHR/CL02</t>
-        </is>
-      </c>
+      <c r="C26" s="15" t="inlineStr"/>
       <c r="D26" s="4" t="n"/>
       <c r="E26" s="11" t="n"/>
       <c r="F26" s="10" t="inlineStr">
@@ -2301,7 +2280,7 @@
         </is>
       </c>
       <c r="C27" s="4" t="n"/>
-      <c r="D27" s="17" t="inlineStr"/>
+      <c r="D27" s="16" t="inlineStr"/>
       <c r="E27" s="11" t="n"/>
       <c r="F27" s="10" t="inlineStr">
         <is>
@@ -2343,15 +2322,15 @@
       <c r="C28" s="4" t="n"/>
       <c r="D28" s="12" t="inlineStr"/>
       <c r="E28" s="11" t="n"/>
-      <c r="F28" s="16" t="inlineStr">
+      <c r="F28" s="15" t="inlineStr">
         <is>
           <t>PB13(CS111)-NAC,SHO/CL05</t>
         </is>
       </c>
       <c r="G28" s="4" t="n"/>
-      <c r="H28" s="10" t="inlineStr">
-        <is>
-          <t>PB14(CS111)-AYS,ANB/CL01</t>
+      <c r="H28" s="14" t="inlineStr">
+        <is>
+          <t>PB14,A10(CS111)-AYS,AM,ANP/CL01,02</t>
         </is>
       </c>
       <c r="I28" s="4" t="n"/>
@@ -2381,9 +2360,9 @@
         </is>
       </c>
       <c r="C29" s="4" t="n"/>
-      <c r="D29" s="17" t="inlineStr"/>
+      <c r="D29" s="16" t="inlineStr"/>
       <c r="E29" s="11" t="n"/>
-      <c r="F29" s="16" t="inlineStr">
+      <c r="F29" s="15" t="inlineStr">
         <is>
           <t>PB14(HS112)-CL12/SDA</t>
         </is>
@@ -2423,17 +2402,13 @@
       <c r="C30" s="4" t="n"/>
       <c r="D30" s="12" t="inlineStr"/>
       <c r="E30" s="11" t="n"/>
-      <c r="F30" s="16" t="inlineStr">
-        <is>
-          <t>PB1(CS111)-AYS,PSO/CL01</t>
+      <c r="F30" s="15" t="inlineStr">
+        <is>
+          <t>PB1,B2(CS111)-AYS,MSI,SLK/CL01,02</t>
         </is>
       </c>
       <c r="G30" s="4" t="n"/>
-      <c r="H30" s="10" t="inlineStr">
-        <is>
-          <t>PA10(CS111)-ANP,VIB/CL02</t>
-        </is>
-      </c>
+      <c r="H30" s="10" t="inlineStr"/>
       <c r="I30" s="4" t="n"/>
       <c r="J30" s="5" t="inlineStr"/>
       <c r="K30" s="1" t="inlineStr"/>
@@ -2463,15 +2438,11 @@
       <c r="C31" s="4" t="n"/>
       <c r="D31" s="12" t="inlineStr"/>
       <c r="E31" s="11" t="n"/>
-      <c r="F31" s="16" t="inlineStr">
-        <is>
-          <t>PB2(CS111)-DCH/SLK/CL02</t>
-        </is>
-      </c>
+      <c r="F31" s="15" t="inlineStr"/>
       <c r="G31" s="4" t="n"/>
-      <c r="H31" s="18" t="inlineStr">
-        <is>
-          <t>PB20(CS111)-MSI,NEH/CL05</t>
+      <c r="H31" s="10" t="inlineStr">
+        <is>
+          <t>PB20(CS111)-DCH,NEH/CL05</t>
         </is>
       </c>
       <c r="I31" s="4" t="n"/>
@@ -2503,7 +2474,7 @@
       <c r="C32" s="4" t="n"/>
       <c r="D32" s="12" t="inlineStr"/>
       <c r="E32" s="11" t="n"/>
-      <c r="F32" s="16" t="inlineStr">
+      <c r="F32" s="15" t="inlineStr">
         <is>
           <t>PB3(EC111)-BEL1/MN.NSH</t>
         </is>
@@ -2543,7 +2514,7 @@
       <c r="C33" s="3" t="n"/>
       <c r="D33" s="4" t="n"/>
       <c r="E33" s="11" t="n"/>
-      <c r="F33" s="16" t="inlineStr">
+      <c r="F33" s="15" t="inlineStr">
         <is>
           <t>PB4(EC111)-BEL2/GRA,CBP</t>
         </is>
@@ -2583,7 +2554,7 @@
       <c r="C34" s="3" t="n"/>
       <c r="D34" s="4" t="n"/>
       <c r="E34" s="11" t="n"/>
-      <c r="F34" s="16" t="inlineStr">
+      <c r="F34" s="15" t="inlineStr">
         <is>
           <t>PB16(EC111)-ADE/BHG,RDR</t>
         </is>
@@ -2722,7 +2693,7 @@
       <c r="Z37" s="1" t="inlineStr"/>
     </row>
     <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="19" t="n"/>
+      <c r="A38" s="17" t="n"/>
       <c r="B38" s="10" t="inlineStr">
         <is>
           <t>PC1(EC112)-EDC/SL,M,RRP</t>
@@ -2730,7 +2701,7 @@
       </c>
       <c r="C38" s="4" t="n"/>
       <c r="D38" s="12" t="inlineStr"/>
-      <c r="E38" s="19" t="n"/>
+      <c r="E38" s="17" t="n"/>
       <c r="F38" s="10" t="inlineStr">
         <is>
           <t>PB8(GE111)-CAD4/ADM</t>
@@ -2758,24 +2729,24 @@
       <c r="Z38" s="1" t="inlineStr"/>
     </row>
     <row r="39" ht="15" customHeight="1">
-      <c r="A39" s="20" t="inlineStr"/>
-      <c r="B39" s="21" t="inlineStr"/>
-      <c r="C39" s="21" t="inlineStr"/>
-      <c r="D39" s="21" t="inlineStr"/>
-      <c r="E39" s="20" t="inlineStr"/>
-      <c r="F39" s="21" t="inlineStr"/>
-      <c r="G39" s="21" t="inlineStr"/>
-      <c r="H39" s="21" t="inlineStr"/>
-      <c r="I39" s="21" t="inlineStr"/>
-      <c r="J39" s="20" t="inlineStr"/>
-      <c r="K39" s="21" t="inlineStr"/>
-      <c r="L39" s="21" t="inlineStr"/>
-      <c r="M39" s="21" t="inlineStr"/>
-      <c r="N39" s="20" t="inlineStr"/>
-      <c r="O39" s="21" t="inlineStr"/>
-      <c r="P39" s="21" t="inlineStr"/>
-      <c r="Q39" s="21" t="inlineStr"/>
-      <c r="R39" s="21" t="inlineStr"/>
+      <c r="A39" s="18" t="inlineStr"/>
+      <c r="B39" s="19" t="inlineStr"/>
+      <c r="C39" s="19" t="inlineStr"/>
+      <c r="D39" s="19" t="inlineStr"/>
+      <c r="E39" s="18" t="inlineStr"/>
+      <c r="F39" s="19" t="inlineStr"/>
+      <c r="G39" s="19" t="inlineStr"/>
+      <c r="H39" s="19" t="inlineStr"/>
+      <c r="I39" s="19" t="inlineStr"/>
+      <c r="J39" s="18" t="inlineStr"/>
+      <c r="K39" s="19" t="inlineStr"/>
+      <c r="L39" s="19" t="inlineStr"/>
+      <c r="M39" s="19" t="inlineStr"/>
+      <c r="N39" s="18" t="inlineStr"/>
+      <c r="O39" s="19" t="inlineStr"/>
+      <c r="P39" s="19" t="inlineStr"/>
+      <c r="Q39" s="19" t="inlineStr"/>
+      <c r="R39" s="19" t="inlineStr"/>
       <c r="S39" s="1" t="inlineStr"/>
       <c r="T39" s="1" t="inlineStr"/>
       <c r="U39" s="1" t="inlineStr"/>
@@ -2922,7 +2893,7 @@
       </c>
       <c r="G42" s="10" t="inlineStr">
         <is>
-          <t>LA15,A16(CI111)-FF2/ROH</t>
+          <t>LA15,A16(CI111)-FF2/RJM</t>
         </is>
       </c>
       <c r="H42" s="10" t="inlineStr">
@@ -2972,11 +2943,7 @@
           <t>LB5,B6(MA111)-FF3/LK</t>
         </is>
       </c>
-      <c r="G43" s="10" t="inlineStr">
-        <is>
-          <t>LB5,B6(CI111)-FF3/RSS</t>
-        </is>
-      </c>
+      <c r="G43" s="12" t="inlineStr"/>
       <c r="H43" s="10" t="inlineStr">
         <is>
           <t>LB5,B6(PH111)-FF3/MKC</t>
@@ -3026,7 +2993,7 @@
       </c>
       <c r="G44" s="10" t="inlineStr">
         <is>
-          <t>LB7,B8(CI111)-FF4/PSO</t>
+          <t>LB7,B8(CI111)-FF4/AW</t>
         </is>
       </c>
       <c r="H44" s="10" t="inlineStr">
@@ -3086,7 +3053,11 @@
           <t>LB11,B12(PH111)-FF8/SDC</t>
         </is>
       </c>
-      <c r="I45" s="12" t="inlineStr"/>
+      <c r="I45" s="10" t="inlineStr">
+        <is>
+          <t>LB5,B6(CI111)-G5/RSS</t>
+        </is>
+      </c>
       <c r="J45" s="5" t="inlineStr"/>
       <c r="K45" s="1" t="inlineStr"/>
       <c r="L45" s="1" t="inlineStr"/>
@@ -3158,14 +3129,10 @@
       <c r="B47" s="12" t="inlineStr"/>
       <c r="C47" s="10" t="inlineStr">
         <is>
-          <t>LG5,G6(CI111)-CS8/SMS</t>
-        </is>
-      </c>
-      <c r="D47" s="10" t="inlineStr">
-        <is>
-          <t>LB1,B2(CI111)-CS8/TNV</t>
-        </is>
-      </c>
+          <t>LG5,G6(CI111)-CS8/PAG</t>
+        </is>
+      </c>
+      <c r="D47" s="12" t="inlineStr"/>
       <c r="E47" s="11" t="n"/>
       <c r="F47" s="10" t="inlineStr">
         <is>
@@ -3407,17 +3374,13 @@
         </is>
       </c>
       <c r="E53" s="11" t="n"/>
-      <c r="F53" s="10" t="inlineStr">
-        <is>
-          <t>TC4(18CI111)-TS6/SJA</t>
-        </is>
-      </c>
+      <c r="F53" s="12" t="inlineStr"/>
       <c r="G53" s="13" t="inlineStr">
         <is>
           <t>TB1(MA111)-TS6//GA</t>
         </is>
       </c>
-      <c r="H53" s="18" t="inlineStr">
+      <c r="H53" s="10" t="inlineStr">
         <is>
           <t>TA7(CI111)-TS6/RCA</t>
         </is>
@@ -3457,7 +3420,7 @@
           <t>TB11(EC111)-TS7/JMO</t>
         </is>
       </c>
-      <c r="D54" s="18" t="inlineStr">
+      <c r="D54" s="10" t="inlineStr">
         <is>
           <t>TB11(CI111)-TS7/AJS</t>
         </is>
@@ -3589,7 +3552,7 @@
       <c r="A57" s="11" t="n"/>
       <c r="B57" s="13" t="inlineStr">
         <is>
-          <t>TB5(CI111)-F7/ROH</t>
+          <t>TB5(CI111)-F7/MAY</t>
         </is>
       </c>
       <c r="C57" s="13" t="inlineStr"/>
@@ -3829,13 +3792,13 @@
       <c r="E63" s="11" t="n"/>
       <c r="F63" s="10" t="inlineStr">
         <is>
-          <t>PB3(CS111)-SMS,MAY/CL01</t>
+          <t>PB3,B4(CS111)-NAC,MAY,RSS/CL01,02</t>
         </is>
       </c>
       <c r="G63" s="4" t="n"/>
       <c r="H63" s="10" t="inlineStr">
         <is>
-          <t>PD1(CS111)-APR,AVR/CL05</t>
+          <t>PD1,G2(CS111)-AVR,ANV,ASA/CL05,06</t>
         </is>
       </c>
       <c r="I63" s="4" t="n"/>
@@ -3867,17 +3830,9 @@
       </c>
       <c r="D64" s="4" t="n"/>
       <c r="E64" s="11" t="n"/>
-      <c r="F64" s="10" t="inlineStr">
-        <is>
-          <t>PB4(CS111)-NAC,SHV/CL02</t>
-        </is>
-      </c>
+      <c r="F64" s="10" t="inlineStr"/>
       <c r="G64" s="4" t="n"/>
-      <c r="H64" s="10" t="inlineStr">
-        <is>
-          <t>PG2(CS111)-ASA,ANV/CL06</t>
-        </is>
-      </c>
+      <c r="H64" s="10" t="inlineStr"/>
       <c r="I64" s="4" t="n"/>
       <c r="J64" s="5" t="inlineStr"/>
       <c r="K64" s="1" t="inlineStr"/>
@@ -3979,9 +3934,9 @@
     </row>
     <row r="67" ht="15.75" customHeight="1">
       <c r="A67" s="11" t="n"/>
-      <c r="B67" s="16" t="inlineStr">
-        <is>
-          <t>PA17(CS111)-DSI,DCH/CL01</t>
+      <c r="B67" s="15" t="inlineStr">
+        <is>
+          <t>PA17,18(CS111)-DCH,SHR,SRG/CL01,02</t>
         </is>
       </c>
       <c r="C67" s="4" t="n"/>
@@ -4019,11 +3974,7 @@
     </row>
     <row r="68" ht="15.75" customHeight="1">
       <c r="A68" s="11" t="n"/>
-      <c r="B68" s="16" t="inlineStr">
-        <is>
-          <t>PA18(CS111)-SHR,SRG/CL02</t>
-        </is>
-      </c>
+      <c r="B68" s="15" t="inlineStr"/>
       <c r="C68" s="4" t="n"/>
       <c r="D68" s="10" t="inlineStr"/>
       <c r="E68" s="11" t="n"/>
@@ -4059,9 +4010,9 @@
     </row>
     <row r="69" ht="15.75" customHeight="1">
       <c r="A69" s="11" t="n"/>
-      <c r="B69" s="16" t="inlineStr">
-        <is>
-          <t>PC4(24CS111)-BS, SHP/CL21</t>
+      <c r="B69" s="20" t="inlineStr">
+        <is>
+          <t>PC4(24CS111)-BS, SHP/CL324</t>
         </is>
       </c>
       <c r="C69" s="4" t="n"/>
@@ -4069,9 +4020,9 @@
       <c r="E69" s="11" t="n"/>
       <c r="F69" s="10" t="inlineStr"/>
       <c r="G69" s="10" t="inlineStr"/>
-      <c r="H69" s="10" t="inlineStr">
-        <is>
-          <t>PC2(24CS111)-BS, MSH/CL21</t>
+      <c r="H69" s="14" t="inlineStr">
+        <is>
+          <t>PC2(24CS111)-BS, MSH/CL306</t>
         </is>
       </c>
       <c r="I69" s="4" t="n"/>
@@ -4110,7 +4061,7 @@
       </c>
       <c r="G70" s="3" t="n"/>
       <c r="H70" s="4" t="n"/>
-      <c r="I70" s="16" t="inlineStr"/>
+      <c r="I70" s="15" t="inlineStr"/>
       <c r="J70" s="5" t="inlineStr"/>
       <c r="K70" s="1" t="inlineStr"/>
       <c r="L70" s="1" t="inlineStr"/>
@@ -4146,7 +4097,7 @@
       </c>
       <c r="G71" s="3" t="n"/>
       <c r="H71" s="4" t="n"/>
-      <c r="I71" s="16" t="inlineStr"/>
+      <c r="I71" s="15" t="inlineStr"/>
       <c r="J71" s="5" t="inlineStr"/>
       <c r="K71" s="1" t="inlineStr"/>
       <c r="L71" s="1" t="inlineStr"/>
@@ -4182,7 +4133,7 @@
       </c>
       <c r="G72" s="3" t="n"/>
       <c r="H72" s="4" t="n"/>
-      <c r="I72" s="16" t="inlineStr"/>
+      <c r="I72" s="15" t="inlineStr"/>
       <c r="J72" s="5" t="inlineStr"/>
       <c r="K72" s="1" t="inlineStr"/>
       <c r="L72" s="1" t="inlineStr"/>
@@ -4218,7 +4169,7 @@
       </c>
       <c r="G73" s="3" t="n"/>
       <c r="H73" s="4" t="n"/>
-      <c r="I73" s="16" t="inlineStr"/>
+      <c r="I73" s="15" t="inlineStr"/>
       <c r="J73" s="5" t="inlineStr"/>
       <c r="K73" s="1" t="inlineStr"/>
       <c r="L73" s="1" t="inlineStr"/>
@@ -4247,10 +4198,10 @@
       <c r="C74" s="3" t="n"/>
       <c r="D74" s="4" t="n"/>
       <c r="E74" s="11" t="n"/>
-      <c r="F74" s="16" t="inlineStr"/>
-      <c r="G74" s="16" t="inlineStr"/>
-      <c r="H74" s="16" t="inlineStr"/>
-      <c r="I74" s="16" t="inlineStr"/>
+      <c r="F74" s="15" t="inlineStr"/>
+      <c r="G74" s="15" t="inlineStr"/>
+      <c r="H74" s="15" t="inlineStr"/>
+      <c r="I74" s="15" t="inlineStr"/>
       <c r="J74" s="5" t="inlineStr"/>
       <c r="K74" s="1" t="inlineStr"/>
       <c r="L74" s="1" t="inlineStr"/>
@@ -4279,9 +4230,9 @@
       <c r="C75" s="3" t="n"/>
       <c r="D75" s="4" t="n"/>
       <c r="E75" s="11" t="n"/>
-      <c r="F75" s="16" t="inlineStr"/>
-      <c r="G75" s="16" t="inlineStr"/>
-      <c r="H75" s="16" t="inlineStr"/>
+      <c r="F75" s="15" t="inlineStr"/>
+      <c r="G75" s="15" t="inlineStr"/>
+      <c r="H75" s="15" t="inlineStr"/>
       <c r="I75" s="13" t="inlineStr"/>
       <c r="J75" s="5" t="inlineStr"/>
       <c r="K75" s="1" t="inlineStr"/>
@@ -4311,9 +4262,9 @@
       <c r="C76" s="3" t="n"/>
       <c r="D76" s="4" t="n"/>
       <c r="E76" s="11" t="n"/>
-      <c r="F76" s="16" t="inlineStr"/>
-      <c r="G76" s="16" t="inlineStr"/>
-      <c r="H76" s="16" t="inlineStr"/>
+      <c r="F76" s="15" t="inlineStr"/>
+      <c r="G76" s="15" t="inlineStr"/>
+      <c r="H76" s="15" t="inlineStr"/>
       <c r="I76" s="13" t="inlineStr"/>
       <c r="J76" s="5" t="inlineStr"/>
       <c r="K76" s="1" t="inlineStr"/>
@@ -4334,7 +4285,7 @@
       <c r="Z76" s="1" t="inlineStr"/>
     </row>
     <row r="77" ht="15" customHeight="1">
-      <c r="A77" s="19" t="n"/>
+      <c r="A77" s="17" t="n"/>
       <c r="B77" s="10" t="inlineStr">
         <is>
           <t>PA6(GE111)-CAD4/NBH</t>
@@ -4342,10 +4293,10 @@
       </c>
       <c r="C77" s="3" t="n"/>
       <c r="D77" s="4" t="n"/>
-      <c r="E77" s="19" t="n"/>
-      <c r="F77" s="16" t="inlineStr"/>
-      <c r="G77" s="16" t="inlineStr"/>
-      <c r="H77" s="16" t="inlineStr"/>
+      <c r="E77" s="17" t="n"/>
+      <c r="F77" s="15" t="inlineStr"/>
+      <c r="G77" s="15" t="inlineStr"/>
+      <c r="H77" s="15" t="inlineStr"/>
       <c r="I77" s="13" t="inlineStr"/>
       <c r="J77" s="5" t="inlineStr"/>
       <c r="K77" s="1" t="inlineStr"/>
@@ -4366,24 +4317,24 @@
       <c r="Z77" s="1" t="inlineStr"/>
     </row>
     <row r="78" ht="15" customHeight="1">
-      <c r="A78" s="20" t="inlineStr"/>
-      <c r="B78" s="21" t="inlineStr"/>
-      <c r="C78" s="21" t="inlineStr"/>
-      <c r="D78" s="21" t="inlineStr"/>
-      <c r="E78" s="20" t="inlineStr"/>
-      <c r="F78" s="21" t="inlineStr"/>
-      <c r="G78" s="21" t="inlineStr"/>
-      <c r="H78" s="21" t="inlineStr"/>
-      <c r="I78" s="21" t="inlineStr"/>
-      <c r="J78" s="20" t="inlineStr"/>
-      <c r="K78" s="21" t="inlineStr"/>
-      <c r="L78" s="21" t="inlineStr"/>
-      <c r="M78" s="21" t="inlineStr"/>
-      <c r="N78" s="20" t="inlineStr"/>
-      <c r="O78" s="21" t="inlineStr"/>
-      <c r="P78" s="21" t="inlineStr"/>
-      <c r="Q78" s="21" t="inlineStr"/>
-      <c r="R78" s="21" t="inlineStr"/>
+      <c r="A78" s="18" t="inlineStr"/>
+      <c r="B78" s="19" t="inlineStr"/>
+      <c r="C78" s="19" t="inlineStr"/>
+      <c r="D78" s="19" t="inlineStr"/>
+      <c r="E78" s="18" t="inlineStr"/>
+      <c r="F78" s="19" t="inlineStr"/>
+      <c r="G78" s="19" t="inlineStr"/>
+      <c r="H78" s="19" t="inlineStr"/>
+      <c r="I78" s="19" t="inlineStr"/>
+      <c r="J78" s="18" t="inlineStr"/>
+      <c r="K78" s="19" t="inlineStr"/>
+      <c r="L78" s="19" t="inlineStr"/>
+      <c r="M78" s="19" t="inlineStr"/>
+      <c r="N78" s="18" t="inlineStr"/>
+      <c r="O78" s="19" t="inlineStr"/>
+      <c r="P78" s="19" t="inlineStr"/>
+      <c r="Q78" s="19" t="inlineStr"/>
+      <c r="R78" s="19" t="inlineStr"/>
       <c r="S78" s="1" t="inlineStr"/>
       <c r="T78" s="1" t="inlineStr"/>
       <c r="U78" s="1" t="inlineStr"/>
@@ -4596,7 +4547,7 @@
       </c>
       <c r="I82" s="10" t="inlineStr">
         <is>
-          <t>LG5,G6(CI111)-FF3/SMS</t>
+          <t>LG5,G6(CI111)-FF3/PAG</t>
         </is>
       </c>
       <c r="J82" s="5" t="inlineStr"/>
@@ -4795,7 +4746,7 @@
       </c>
       <c r="H86" s="10" t="inlineStr">
         <is>
-          <t>LG1,G2(CI111)-FF9/VIB</t>
+          <t>LG1,G2(CI111)-FF9/DSI</t>
         </is>
       </c>
       <c r="I86" s="12" t="inlineStr"/>
@@ -4864,7 +4815,7 @@
     <row r="88" ht="15.75" customHeight="1">
       <c r="A88" s="11" t="n"/>
       <c r="B88" s="10" t="inlineStr"/>
-      <c r="C88" s="14" t="inlineStr"/>
+      <c r="C88" s="12" t="inlineStr"/>
       <c r="D88" s="10" t="inlineStr">
         <is>
           <t>LA7,A8(MA111)-CS8/NF1</t>
@@ -4876,7 +4827,7 @@
           <t>LB15,B16(CI111)-G8/NAC</t>
         </is>
       </c>
-      <c r="G88" s="14" t="inlineStr"/>
+      <c r="G88" s="12" t="inlineStr"/>
       <c r="H88" s="12" t="inlineStr"/>
       <c r="I88" s="12" t="inlineStr"/>
       <c r="J88" s="5" t="inlineStr"/>
@@ -4912,7 +4863,7 @@
           <t>LC1,C2,C3(PH112)-G9/DAM</t>
         </is>
       </c>
-      <c r="G89" s="18" t="inlineStr"/>
+      <c r="G89" s="10" t="inlineStr"/>
       <c r="H89" s="12" t="inlineStr"/>
       <c r="I89" s="12" t="inlineStr"/>
       <c r="J89" s="5" t="inlineStr"/>
@@ -4952,7 +4903,7 @@
       </c>
       <c r="E90" s="11" t="n"/>
       <c r="F90" s="12" t="inlineStr"/>
-      <c r="G90" s="14" t="inlineStr"/>
+      <c r="G90" s="12" t="inlineStr"/>
       <c r="H90" s="10" t="inlineStr">
         <is>
           <t>TB3(MA111)-TS6/HPT</t>
@@ -5045,7 +4996,7 @@
       <c r="E92" s="11" t="n"/>
       <c r="F92" s="10" t="inlineStr">
         <is>
-          <t>TG6(CI111)-TS6/ROH</t>
+          <t>TG6(CI111)-TS6/IC</t>
         </is>
       </c>
       <c r="G92" s="10" t="inlineStr">
@@ -5060,7 +5011,7 @@
       </c>
       <c r="I92" s="13" t="inlineStr">
         <is>
-          <t>TB2(CI111)-TS7/PSO</t>
+          <t>TB2(CI111)-TS7/APR</t>
         </is>
       </c>
       <c r="J92" s="5" t="inlineStr"/>
@@ -5195,7 +5146,7 @@
       </c>
       <c r="D95" s="13" t="inlineStr">
         <is>
-          <t>TA18(CI111)-TR307/PSO</t>
+          <t>TA18(CI111)-TR307/SRG</t>
         </is>
       </c>
       <c r="E95" s="11" t="n"/>
@@ -5383,9 +5334,9 @@
       </c>
       <c r="D100" s="4" t="n"/>
       <c r="E100" s="11" t="n"/>
-      <c r="F100" s="22" t="inlineStr">
-        <is>
-          <t>PH1(CS111)-SHV,PTK/CL03</t>
+      <c r="F100" s="15" t="inlineStr">
+        <is>
+          <t>PH1(CS111)-SLK,PTK/CL03</t>
         </is>
       </c>
       <c r="G100" s="4" t="n"/>
@@ -5419,7 +5370,7 @@
       </c>
       <c r="D101" s="4" t="n"/>
       <c r="E101" s="11" t="n"/>
-      <c r="F101" s="16" t="inlineStr">
+      <c r="F101" s="15" t="inlineStr">
         <is>
           <t>PH2(PH171)-PL1/NKS</t>
         </is>
@@ -5459,7 +5410,7 @@
       </c>
       <c r="D102" s="4" t="n"/>
       <c r="E102" s="11" t="n"/>
-      <c r="F102" s="16" t="inlineStr">
+      <c r="F102" s="15" t="inlineStr">
         <is>
           <t>PB1(PH171)-PL2/MTR</t>
         </is>
@@ -5499,7 +5450,7 @@
       </c>
       <c r="D103" s="4" t="n"/>
       <c r="E103" s="11" t="n"/>
-      <c r="F103" s="16" t="inlineStr">
+      <c r="F103" s="15" t="inlineStr">
         <is>
           <t>PB2(PH171)-PL3/NG</t>
         </is>
@@ -5539,7 +5490,7 @@
       </c>
       <c r="D104" s="4" t="n"/>
       <c r="E104" s="11" t="n"/>
-      <c r="F104" s="16" t="inlineStr">
+      <c r="F104" s="15" t="inlineStr">
         <is>
           <t>PA1(HS112)-CL12/SDA</t>
         </is>
@@ -5579,7 +5530,7 @@
       </c>
       <c r="D105" s="4" t="n"/>
       <c r="E105" s="11" t="n"/>
-      <c r="F105" s="16" t="inlineStr">
+      <c r="F105" s="15" t="inlineStr">
         <is>
           <t>PA2(HS112)- LL/KMB</t>
         </is>
@@ -5619,15 +5570,15 @@
       </c>
       <c r="D106" s="4" t="n"/>
       <c r="E106" s="11" t="n"/>
-      <c r="F106" s="16" t="inlineStr">
-        <is>
-          <t>PA3(CS111)-AYS,DCH/CL01</t>
+      <c r="F106" s="15" t="inlineStr">
+        <is>
+          <t>PA3,A4(CS111)-AYS,DCH,MAY/CL01,02</t>
         </is>
       </c>
       <c r="G106" s="4" t="n"/>
       <c r="H106" s="10" t="inlineStr">
         <is>
-          <t>PA5(CS111)-AW, ASA/CL05</t>
+          <t>PA5,A6(CS111)-AW, ASA/CL05</t>
         </is>
       </c>
       <c r="I106" s="4" t="n"/>
@@ -5654,12 +5605,12 @@
       <c r="B107" s="13" t="inlineStr"/>
       <c r="C107" s="10" t="inlineStr">
         <is>
-          <t>PB10(CS111)-ANV,DSI/CL07</t>
+          <t>PB10(CS111)-PAG,DSI/CL07</t>
         </is>
       </c>
       <c r="D107" s="4" t="n"/>
       <c r="E107" s="11" t="n"/>
-      <c r="F107" s="16" t="inlineStr">
+      <c r="F107" s="15" t="inlineStr">
         <is>
           <t>PD3(HS112)-LL1/MDU</t>
         </is>
@@ -5699,13 +5650,9 @@
       <c r="C108" s="4" t="n"/>
       <c r="D108" s="10" t="inlineStr"/>
       <c r="E108" s="11" t="n"/>
-      <c r="F108" s="16" t="inlineStr">
-        <is>
-          <t>PA4(CS111)-MAY, AM/CL02</t>
-        </is>
-      </c>
+      <c r="F108" s="15" t="inlineStr"/>
       <c r="G108" s="4" t="n"/>
-      <c r="H108" s="18" t="inlineStr">
+      <c r="H108" s="10" t="inlineStr">
         <is>
           <t>PB16(CS111)-AKT,SHO/ CL06</t>
         </is>
@@ -5739,7 +5686,7 @@
       <c r="C109" s="4" t="n"/>
       <c r="D109" s="10" t="inlineStr"/>
       <c r="E109" s="11" t="n"/>
-      <c r="F109" s="16" t="inlineStr">
+      <c r="F109" s="15" t="inlineStr">
         <is>
           <t>PG1(EC111)-BEL1/MN,NSH</t>
         </is>
@@ -5779,7 +5726,7 @@
       <c r="C110" s="4" t="n"/>
       <c r="D110" s="10" t="inlineStr"/>
       <c r="E110" s="11" t="n"/>
-      <c r="F110" s="16" t="inlineStr">
+      <c r="F110" s="15" t="inlineStr">
         <is>
           <t>PG2(EC111)-BEL2/BHG,VSS</t>
         </is>
@@ -5815,7 +5762,7 @@
       <c r="C111" s="12" t="inlineStr"/>
       <c r="D111" s="10" t="inlineStr"/>
       <c r="E111" s="11" t="n"/>
-      <c r="F111" s="16" t="inlineStr">
+      <c r="F111" s="15" t="inlineStr">
         <is>
           <t>PD4(EC111)-EDC/ATA,BVI</t>
         </is>
@@ -5855,7 +5802,7 @@
       <c r="C112" s="3" t="n"/>
       <c r="D112" s="4" t="n"/>
       <c r="E112" s="11" t="n"/>
-      <c r="F112" s="16" t="inlineStr">
+      <c r="F112" s="15" t="inlineStr">
         <is>
           <t>PC5(EC112)-ADE/RRJ,SIM</t>
         </is>
@@ -5990,7 +5937,7 @@
       <c r="Z115" s="1" t="inlineStr"/>
     </row>
     <row r="116" ht="15.75" customHeight="1">
-      <c r="A116" s="19" t="n"/>
+      <c r="A116" s="17" t="n"/>
       <c r="B116" s="10" t="inlineStr">
         <is>
           <t>PG3(GE111)-CAD4/CDN</t>
@@ -5998,7 +5945,7 @@
       </c>
       <c r="C116" s="3" t="n"/>
       <c r="D116" s="4" t="n"/>
-      <c r="E116" s="19" t="n"/>
+      <c r="E116" s="17" t="n"/>
       <c r="F116" s="10" t="inlineStr">
         <is>
           <t>PA8(GE111)-CAD4/ASG</t>
@@ -6026,24 +5973,24 @@
       <c r="Z116" s="1" t="inlineStr"/>
     </row>
     <row r="117" ht="7.5" customHeight="1">
-      <c r="A117" s="20" t="inlineStr"/>
-      <c r="B117" s="21" t="inlineStr"/>
-      <c r="C117" s="21" t="inlineStr"/>
-      <c r="D117" s="21" t="inlineStr"/>
-      <c r="E117" s="20" t="inlineStr"/>
-      <c r="F117" s="21" t="inlineStr"/>
-      <c r="G117" s="21" t="inlineStr"/>
-      <c r="H117" s="21" t="inlineStr"/>
-      <c r="I117" s="21" t="inlineStr"/>
-      <c r="J117" s="20" t="inlineStr"/>
-      <c r="K117" s="21" t="inlineStr"/>
-      <c r="L117" s="21" t="inlineStr"/>
-      <c r="M117" s="21" t="inlineStr"/>
-      <c r="N117" s="20" t="inlineStr"/>
-      <c r="O117" s="21" t="inlineStr"/>
-      <c r="P117" s="21" t="inlineStr"/>
-      <c r="Q117" s="21" t="inlineStr"/>
-      <c r="R117" s="21" t="inlineStr"/>
+      <c r="A117" s="18" t="inlineStr"/>
+      <c r="B117" s="19" t="inlineStr"/>
+      <c r="C117" s="19" t="inlineStr"/>
+      <c r="D117" s="19" t="inlineStr"/>
+      <c r="E117" s="18" t="inlineStr"/>
+      <c r="F117" s="19" t="inlineStr"/>
+      <c r="G117" s="19" t="inlineStr"/>
+      <c r="H117" s="19" t="inlineStr"/>
+      <c r="I117" s="19" t="inlineStr"/>
+      <c r="J117" s="18" t="inlineStr"/>
+      <c r="K117" s="19" t="inlineStr"/>
+      <c r="L117" s="19" t="inlineStr"/>
+      <c r="M117" s="19" t="inlineStr"/>
+      <c r="N117" s="18" t="inlineStr"/>
+      <c r="O117" s="19" t="inlineStr"/>
+      <c r="P117" s="19" t="inlineStr"/>
+      <c r="Q117" s="19" t="inlineStr"/>
+      <c r="R117" s="19" t="inlineStr"/>
       <c r="S117" s="1" t="inlineStr"/>
       <c r="T117" s="1" t="inlineStr"/>
       <c r="U117" s="1" t="inlineStr"/>
@@ -6183,7 +6130,7 @@
       </c>
       <c r="D120" s="10" t="inlineStr">
         <is>
-          <t>LA15,A16(CI111)-FF2/ROH</t>
+          <t>LA15,A16(CI111)-FF2/RJM</t>
         </is>
       </c>
       <c r="E120" s="11" t="n"/>
@@ -6204,7 +6151,7 @@
       </c>
       <c r="I120" s="10" t="inlineStr">
         <is>
-          <t>LH1,H2(CI111)-FF2/SHV</t>
+          <t>LH1,H2(CI111)-FF2/AW</t>
         </is>
       </c>
       <c r="J120" s="5" t="inlineStr"/>
@@ -6287,7 +6234,7 @@
       </c>
       <c r="D122" s="10" t="inlineStr">
         <is>
-          <t>LB7,B8(CI111)-FF4/PSO</t>
+          <t>LB7,B8(CI111)-FF4/AW</t>
         </is>
       </c>
       <c r="E122" s="11" t="n"/>
@@ -6511,7 +6458,7 @@
       </c>
       <c r="D127" s="10" t="inlineStr">
         <is>
-          <t>LG1,G2(CI111)-CS8/VIB</t>
+          <t>LG1,G2(CI111)-CS8/DSI</t>
         </is>
       </c>
       <c r="E127" s="11" t="n"/>
@@ -6900,9 +6847,9 @@
     <row r="136" ht="15.75" customHeight="1">
       <c r="A136" s="11" t="n"/>
       <c r="B136" s="12" t="inlineStr"/>
-      <c r="C136" s="16" t="inlineStr">
-        <is>
-          <t>PD3(CS111)-SLK, MSI/CL01</t>
+      <c r="C136" s="15" t="inlineStr">
+        <is>
+          <t>PA1,D3(CS111)-TAJ,ANP,AM/CL01,02</t>
         </is>
       </c>
       <c r="D136" s="4" t="n"/>
@@ -6914,12 +6861,12 @@
       </c>
       <c r="G136" s="10" t="inlineStr">
         <is>
-          <t>TG2(CI111)-TR326/SHV</t>
-        </is>
-      </c>
-      <c r="H136" s="16" t="inlineStr">
-        <is>
-          <t>PC5(24CS111)-MSH, SJA/CL05</t>
+          <t>TG2(CI111)-TR326/IC</t>
+        </is>
+      </c>
+      <c r="H136" s="15" t="inlineStr">
+        <is>
+          <t>PC5(24CS111)-MSH,SJA/CL05</t>
         </is>
       </c>
       <c r="I136" s="4" t="n"/>
@@ -6944,7 +6891,7 @@
     <row r="137" ht="15.75" customHeight="1">
       <c r="A137" s="11" t="n"/>
       <c r="B137" s="1" t="inlineStr"/>
-      <c r="C137" s="16" t="inlineStr">
+      <c r="C137" s="15" t="inlineStr">
         <is>
           <t>PA3(PH171)-PL1/RAV</t>
         </is>
@@ -6984,7 +6931,7 @@
     <row r="138" ht="15.75" customHeight="1">
       <c r="A138" s="11" t="n"/>
       <c r="B138" s="1" t="inlineStr"/>
-      <c r="C138" s="16" t="inlineStr">
+      <c r="C138" s="15" t="inlineStr">
         <is>
           <t>PC4(PH171)Pl2/DAM</t>
         </is>
@@ -7024,7 +6971,7 @@
     <row r="139" ht="15.75" customHeight="1">
       <c r="A139" s="11" t="n"/>
       <c r="B139" s="1" t="inlineStr"/>
-      <c r="C139" s="16" t="inlineStr">
+      <c r="C139" s="15" t="inlineStr">
         <is>
           <t>PC2(PH171)-PL3/EKY</t>
         </is>
@@ -7064,7 +7011,7 @@
     <row r="140" ht="15.75" customHeight="1">
       <c r="A140" s="11" t="n"/>
       <c r="B140" s="12" t="inlineStr"/>
-      <c r="C140" s="16" t="inlineStr">
+      <c r="C140" s="15" t="inlineStr">
         <is>
           <t>PB20(HS112)-CL12/KNP</t>
         </is>
@@ -7104,7 +7051,7 @@
     <row r="141" ht="15.75" customHeight="1">
       <c r="A141" s="11" t="n"/>
       <c r="B141" s="1" t="inlineStr"/>
-      <c r="C141" s="16" t="inlineStr">
+      <c r="C141" s="15" t="inlineStr">
         <is>
           <t>PA8(HS112)-LL1/NIS</t>
         </is>
@@ -7144,11 +7091,7 @@
     <row r="142" ht="15.75" customHeight="1">
       <c r="A142" s="11" t="n"/>
       <c r="B142" s="1" t="inlineStr"/>
-      <c r="C142" s="16" t="inlineStr">
-        <is>
-          <t>PA1(CS111)-TAJ, AM/CL02</t>
-        </is>
-      </c>
+      <c r="C142" s="15" t="inlineStr"/>
       <c r="D142" s="4" t="n"/>
       <c r="E142" s="11" t="n"/>
       <c r="F142" s="10" t="inlineStr">
@@ -7191,15 +7134,15 @@
       </c>
       <c r="D143" s="4" t="n"/>
       <c r="E143" s="11" t="n"/>
-      <c r="F143" s="10" t="inlineStr">
-        <is>
-          <t>PB11(CS111)-PSO,ANP/CL05</t>
+      <c r="F143" s="14" t="inlineStr">
+        <is>
+          <t>PB11,B12(CS111)-ANB,RCA,ANP/CL05,06</t>
         </is>
       </c>
       <c r="G143" s="4" t="n"/>
       <c r="H143" s="10" t="inlineStr">
         <is>
-          <t>PA8(CS111)-SAA,ROH/CL01</t>
+          <t>PA8(CS111)-SAA,ANV/CL01</t>
         </is>
       </c>
       <c r="I143" s="4" t="n"/>
@@ -7231,11 +7174,7 @@
       <c r="C144" s="12" t="inlineStr"/>
       <c r="D144" s="12" t="inlineStr"/>
       <c r="E144" s="11" t="n"/>
-      <c r="F144" s="10" t="inlineStr">
-        <is>
-          <t>PB12(CS111)-RJM,RCA/CL06</t>
-        </is>
-      </c>
+      <c r="F144" s="10" t="inlineStr"/>
       <c r="G144" s="4" t="n"/>
       <c r="H144" s="10" t="inlineStr">
         <is>
@@ -7263,9 +7202,9 @@
     </row>
     <row r="145" ht="15.75" customHeight="1">
       <c r="A145" s="11" t="n"/>
-      <c r="B145" s="16" t="inlineStr">
-        <is>
-          <t>PC1(24CS111)-SHP, BS/CL21</t>
+      <c r="B145" s="20" t="inlineStr">
+        <is>
+          <t>PC1(24CS111)-SHP, BS/CL306</t>
         </is>
       </c>
       <c r="C145" s="4" t="n"/>
@@ -7383,9 +7322,9 @@
     </row>
     <row r="148" ht="15.75" customHeight="1">
       <c r="A148" s="11" t="n"/>
-      <c r="B148" s="16" t="inlineStr">
-        <is>
-          <t>PA2(CS111)-SAA,ROH/CL05</t>
+      <c r="B148" s="15" t="inlineStr">
+        <is>
+          <t>PA2(CS111)-SAA,RCA/CL05</t>
         </is>
       </c>
       <c r="C148" s="4" t="n"/>
@@ -7554,7 +7493,7 @@
       <c r="Z152" s="1" t="inlineStr"/>
     </row>
     <row r="153" ht="15.75" customHeight="1">
-      <c r="A153" s="19" t="n"/>
+      <c r="A153" s="17" t="n"/>
       <c r="B153" s="10" t="inlineStr">
         <is>
           <t>PC5(GE111)-SPL/CDN</t>
@@ -7562,7 +7501,7 @@
       </c>
       <c r="C153" s="3" t="n"/>
       <c r="D153" s="4" t="n"/>
-      <c r="E153" s="19" t="n"/>
+      <c r="E153" s="17" t="n"/>
       <c r="F153" s="10" t="inlineStr">
         <is>
           <t>PG4(GE111)-CAD4/MJH</t>
@@ -7590,24 +7529,24 @@
       <c r="Z153" s="1" t="inlineStr"/>
     </row>
     <row r="154" ht="6" customHeight="1">
-      <c r="A154" s="20" t="inlineStr"/>
-      <c r="B154" s="21" t="inlineStr"/>
-      <c r="C154" s="21" t="inlineStr"/>
-      <c r="D154" s="21" t="inlineStr"/>
-      <c r="E154" s="20" t="inlineStr"/>
-      <c r="F154" s="21" t="inlineStr"/>
-      <c r="G154" s="21" t="inlineStr"/>
-      <c r="H154" s="21" t="inlineStr"/>
-      <c r="I154" s="21" t="inlineStr"/>
-      <c r="J154" s="20" t="inlineStr"/>
-      <c r="K154" s="21" t="inlineStr"/>
-      <c r="L154" s="21" t="inlineStr"/>
-      <c r="M154" s="21" t="inlineStr"/>
-      <c r="N154" s="20" t="inlineStr"/>
-      <c r="O154" s="21" t="inlineStr"/>
-      <c r="P154" s="21" t="inlineStr"/>
-      <c r="Q154" s="21" t="inlineStr"/>
-      <c r="R154" s="21" t="inlineStr"/>
+      <c r="A154" s="18" t="inlineStr"/>
+      <c r="B154" s="19" t="inlineStr"/>
+      <c r="C154" s="19" t="inlineStr"/>
+      <c r="D154" s="19" t="inlineStr"/>
+      <c r="E154" s="18" t="inlineStr"/>
+      <c r="F154" s="19" t="inlineStr"/>
+      <c r="G154" s="19" t="inlineStr"/>
+      <c r="H154" s="19" t="inlineStr"/>
+      <c r="I154" s="19" t="inlineStr"/>
+      <c r="J154" s="18" t="inlineStr"/>
+      <c r="K154" s="19" t="inlineStr"/>
+      <c r="L154" s="19" t="inlineStr"/>
+      <c r="M154" s="19" t="inlineStr"/>
+      <c r="N154" s="18" t="inlineStr"/>
+      <c r="O154" s="19" t="inlineStr"/>
+      <c r="P154" s="19" t="inlineStr"/>
+      <c r="Q154" s="19" t="inlineStr"/>
+      <c r="R154" s="19" t="inlineStr"/>
       <c r="S154" s="1" t="inlineStr"/>
       <c r="T154" s="1" t="inlineStr"/>
       <c r="U154" s="1" t="inlineStr"/>
@@ -7660,7 +7599,7 @@
       </c>
       <c r="I155" s="13" t="inlineStr">
         <is>
-          <t>LH1,H2(CI111)-G1/SHV</t>
+          <t>LH1,H2(CI111)-G1/AW</t>
         </is>
       </c>
       <c r="J155" s="5" t="inlineStr"/>
@@ -7930,7 +7869,11 @@
           <t>LG1,G2(EC111)-G6/VSS</t>
         </is>
       </c>
-      <c r="I160" s="12" t="inlineStr"/>
+      <c r="I160" s="14" t="inlineStr">
+        <is>
+          <t>TB10(CI111)-TR302/APR</t>
+        </is>
+      </c>
       <c r="J160" s="5" t="inlineStr"/>
       <c r="K160" s="1" t="inlineStr"/>
       <c r="L160" s="1" t="inlineStr"/>
@@ -8055,7 +7998,7 @@
       </c>
       <c r="D163" s="13" t="inlineStr">
         <is>
-          <t>LG1,G2(CI111)-CS7/VIB</t>
+          <t>LG1,G2(CI111)-CS7/DSI</t>
         </is>
       </c>
       <c r="E163" s="11" t="n"/>
@@ -8165,7 +8108,7 @@
       <c r="E166" s="11" t="n"/>
       <c r="F166" s="13" t="inlineStr">
         <is>
-          <t>TB16(CI111)-TS6/AYS</t>
+          <t>TB16(CI111)-TS6/IC</t>
         </is>
       </c>
       <c r="G166" s="10" t="inlineStr">
@@ -8203,11 +8146,7 @@
     </row>
     <row r="167" ht="15.75" customHeight="1">
       <c r="A167" s="11" t="n"/>
-      <c r="B167" s="10" t="inlineStr">
-        <is>
-          <t>TB10(CI111)-TS6SHV</t>
-        </is>
-      </c>
+      <c r="B167" s="12" t="inlineStr"/>
       <c r="C167" s="10" t="inlineStr">
         <is>
           <t>TA1(MA111)-TS6/NS</t>
@@ -8283,7 +8222,7 @@
       </c>
       <c r="H168" s="10" t="inlineStr">
         <is>
-          <t>TA15(CI111)-TS8/PKU</t>
+          <t>TA15(CI111)-TS8/AYS</t>
         </is>
       </c>
       <c r="I168" s="13" t="inlineStr">
@@ -8329,7 +8268,7 @@
       <c r="E169" s="11" t="n"/>
       <c r="F169" s="13" t="inlineStr">
         <is>
-          <t>TB6(CI111)-F4/SHV</t>
+          <t>TB6(CI111)-F4/SRG</t>
         </is>
       </c>
       <c r="G169" s="13" t="inlineStr">
@@ -8425,7 +8364,11 @@
           <t>TH2(PH111)-F7/MTR</t>
         </is>
       </c>
-      <c r="D171" s="12" t="inlineStr"/>
+      <c r="D171" s="10" t="inlineStr">
+        <is>
+          <t>TC4(18CI111)-TR307/SJA</t>
+        </is>
+      </c>
       <c r="E171" s="11" t="n"/>
       <c r="F171" s="13" t="inlineStr">
         <is>
@@ -8571,11 +8514,11 @@
       </c>
       <c r="D175" s="4" t="n"/>
       <c r="E175" s="11" t="n"/>
-      <c r="F175" s="16" t="inlineStr"/>
+      <c r="F175" s="15" t="inlineStr"/>
       <c r="G175" s="4" t="n"/>
-      <c r="H175" s="18" t="inlineStr">
-        <is>
-          <t>PB15(CS111)-ANP,AM/CL01</t>
+      <c r="H175" s="10" t="inlineStr">
+        <is>
+          <t>PB15,D4(CS111)-MSI,DCH,NAC/CL01,02</t>
         </is>
       </c>
       <c r="I175" s="4" t="n"/>
@@ -8761,7 +8704,7 @@
       <c r="A180" s="11" t="n"/>
       <c r="B180" s="12" t="inlineStr"/>
       <c r="C180" s="12" t="inlineStr"/>
-      <c r="D180" s="17" t="inlineStr"/>
+      <c r="D180" s="16" t="inlineStr"/>
       <c r="E180" s="11" t="n"/>
       <c r="F180" s="10" t="inlineStr">
         <is>
@@ -8771,7 +8714,7 @@
       <c r="G180" s="4" t="n"/>
       <c r="H180" s="10" t="inlineStr">
         <is>
-          <t>PB7(CS111)-SOS,NEH/CL05</t>
+          <t>PB7,B8(CS111)-SOS,NEH,NIY/CL05,06</t>
         </is>
       </c>
       <c r="I180" s="4" t="n"/>
@@ -8809,11 +8752,7 @@
         </is>
       </c>
       <c r="G181" s="4" t="n"/>
-      <c r="H181" s="10" t="inlineStr">
-        <is>
-          <t>PB8(CS111)-SMS,NIY/CL06</t>
-        </is>
-      </c>
+      <c r="H181" s="10" t="inlineStr"/>
       <c r="I181" s="4" t="n"/>
       <c r="J181" s="5" t="inlineStr"/>
       <c r="K181" s="1" t="inlineStr"/>
@@ -8845,15 +8784,11 @@
       <c r="E182" s="11" t="n"/>
       <c r="F182" s="10" t="inlineStr">
         <is>
-          <t>PA15(CS111)-RSS,SOS/CL03</t>
+          <t>PA15,A16(CS111)-ANP,SOS,PKU/CL02,03</t>
         </is>
       </c>
       <c r="G182" s="4" t="n"/>
-      <c r="H182" s="18" t="inlineStr">
-        <is>
-          <t>PD4(CS111)-DCH,NAC/CL02</t>
-        </is>
-      </c>
+      <c r="H182" s="10" t="inlineStr"/>
       <c r="I182" s="4" t="n"/>
       <c r="J182" s="5" t="inlineStr"/>
       <c r="K182" s="1" t="inlineStr"/>
@@ -8883,11 +8818,7 @@
       <c r="C183" s="3" t="n"/>
       <c r="D183" s="4" t="n"/>
       <c r="E183" s="11" t="n"/>
-      <c r="F183" s="16" t="inlineStr">
-        <is>
-          <t>PA16(CS111)-ANP,PKU/CL02</t>
-        </is>
-      </c>
+      <c r="F183" s="15" t="inlineStr"/>
       <c r="G183" s="4" t="n"/>
       <c r="H183" s="12" t="inlineStr"/>
       <c r="I183" s="12" t="inlineStr"/>
@@ -8947,7 +8878,7 @@
     </row>
     <row r="185" ht="15.75" customHeight="1">
       <c r="A185" s="11" t="n"/>
-      <c r="B185" s="16" t="inlineStr">
+      <c r="B185" s="15" t="inlineStr">
         <is>
           <t>PC3(24CS111)-APR, SJA/CL01</t>
         </is>
@@ -9026,7 +8957,7 @@
       </c>
       <c r="G187" s="3" t="n"/>
       <c r="H187" s="4" t="n"/>
-      <c r="I187" s="16" t="inlineStr"/>
+      <c r="I187" s="15" t="inlineStr"/>
       <c r="J187" s="5" t="inlineStr"/>
       <c r="K187" s="1" t="inlineStr"/>
       <c r="L187" s="1" t="inlineStr"/>
@@ -9046,11 +8977,11 @@
       <c r="Z187" s="1" t="inlineStr"/>
     </row>
     <row r="188" ht="15.75" customHeight="1">
-      <c r="A188" s="19" t="n"/>
+      <c r="A188" s="17" t="n"/>
       <c r="B188" s="12" t="inlineStr"/>
       <c r="C188" s="12" t="inlineStr"/>
       <c r="D188" s="12" t="inlineStr"/>
-      <c r="E188" s="19" t="n"/>
+      <c r="E188" s="17" t="n"/>
       <c r="F188" s="10" t="inlineStr">
         <is>
           <t>PA17(GE111)-CAD4/NBH</t>
@@ -9078,24 +9009,24 @@
       <c r="Z188" s="1" t="inlineStr"/>
     </row>
     <row r="189" ht="6.75" customHeight="1">
-      <c r="A189" s="20" t="inlineStr"/>
-      <c r="B189" s="21" t="inlineStr"/>
-      <c r="C189" s="21" t="inlineStr"/>
-      <c r="D189" s="21" t="inlineStr"/>
-      <c r="E189" s="20" t="inlineStr"/>
-      <c r="F189" s="21" t="inlineStr"/>
-      <c r="G189" s="21" t="inlineStr"/>
-      <c r="H189" s="21" t="inlineStr"/>
-      <c r="I189" s="21" t="inlineStr"/>
-      <c r="J189" s="20" t="inlineStr"/>
-      <c r="K189" s="21" t="inlineStr"/>
-      <c r="L189" s="21" t="inlineStr"/>
-      <c r="M189" s="21" t="inlineStr"/>
-      <c r="N189" s="20" t="inlineStr"/>
-      <c r="O189" s="21" t="inlineStr"/>
-      <c r="P189" s="21" t="inlineStr"/>
-      <c r="Q189" s="21" t="inlineStr"/>
-      <c r="R189" s="21" t="inlineStr"/>
+      <c r="A189" s="18" t="inlineStr"/>
+      <c r="B189" s="19" t="inlineStr"/>
+      <c r="C189" s="19" t="inlineStr"/>
+      <c r="D189" s="19" t="inlineStr"/>
+      <c r="E189" s="18" t="inlineStr"/>
+      <c r="F189" s="19" t="inlineStr"/>
+      <c r="G189" s="19" t="inlineStr"/>
+      <c r="H189" s="19" t="inlineStr"/>
+      <c r="I189" s="19" t="inlineStr"/>
+      <c r="J189" s="18" t="inlineStr"/>
+      <c r="K189" s="19" t="inlineStr"/>
+      <c r="L189" s="19" t="inlineStr"/>
+      <c r="M189" s="19" t="inlineStr"/>
+      <c r="N189" s="18" t="inlineStr"/>
+      <c r="O189" s="19" t="inlineStr"/>
+      <c r="P189" s="19" t="inlineStr"/>
+      <c r="Q189" s="19" t="inlineStr"/>
+      <c r="R189" s="19" t="inlineStr"/>
       <c r="S189" s="1" t="inlineStr"/>
       <c r="T189" s="1" t="inlineStr"/>
       <c r="U189" s="1" t="inlineStr"/>
@@ -9111,7 +9042,7 @@
           <t>SAT</t>
         </is>
       </c>
-      <c r="B190" s="23" t="inlineStr">
+      <c r="B190" s="21" t="inlineStr">
         <is>
           <t>LH1,H2(PH111)-G6/RAV</t>
         </is>
@@ -9121,12 +9052,12 @@
           <t>LA3,A4(EC111)-G1/BVI,SHWETA</t>
         </is>
       </c>
-      <c r="D190" s="23" t="inlineStr">
+      <c r="D190" s="21" t="inlineStr">
         <is>
           <t>LA5,A6(MA111)-G1/RSA</t>
         </is>
       </c>
-      <c r="E190" s="23" t="inlineStr">
+      <c r="E190" s="21" t="inlineStr">
         <is>
           <t>LA10,B20(EC111)-G1/VGO</t>
         </is>
@@ -9251,7 +9182,7 @@
       </c>
       <c r="D193" s="13" t="inlineStr">
         <is>
-          <t>LH1,H2(CI111)-FF3/SHV</t>
+          <t>LH1,H2(CI111)-FF3/AW</t>
         </is>
       </c>
       <c r="E193" s="12" t="inlineStr"/>
@@ -9318,7 +9249,7 @@
       <c r="B195" s="12" t="inlineStr"/>
       <c r="C195" s="13" t="inlineStr">
         <is>
-          <t>LB7,B8(CI111)-G3/PSO</t>
+          <t>LB7,B8(CI111)-G3/AW</t>
         </is>
       </c>
       <c r="D195" s="13" t="inlineStr">
@@ -9464,7 +9395,7 @@
       </c>
       <c r="E199" s="13" t="inlineStr">
         <is>
-          <t>TD3(CI111)-TS6/ROH</t>
+          <t>TD3(CI111)-TS6/SHR</t>
         </is>
       </c>
       <c r="F199" s="1" t="inlineStr"/>
@@ -9685,7 +9616,7 @@
       <c r="A205" s="11" t="n"/>
       <c r="B205" s="10" t="inlineStr">
         <is>
-          <t>TA3(CI111)-TS16/AYS</t>
+          <t>TA3(CI111)-TS16/SHR</t>
         </is>
       </c>
       <c r="C205" s="10" t="inlineStr"/>
@@ -9859,7 +9790,7 @@
       <c r="C210" s="4" t="n"/>
       <c r="D210" s="10" t="inlineStr">
         <is>
-          <t>PG1(CS111)-ANV,ANB/CL01</t>
+          <t>PG1,D2(CS111)-ANV,ANB,TAJ/CL01,02</t>
         </is>
       </c>
       <c r="E210" s="4" t="n"/>
@@ -9893,11 +9824,7 @@
         </is>
       </c>
       <c r="C211" s="4" t="n"/>
-      <c r="D211" s="10" t="inlineStr">
-        <is>
-          <t>PD2(CS111)-TAJ,RSS/CL03</t>
-        </is>
-      </c>
+      <c r="D211" s="10" t="inlineStr"/>
       <c r="E211" s="4" t="n"/>
       <c r="F211" s="10" t="inlineStr"/>
       <c r="G211" s="10" t="inlineStr"/>
@@ -10029,7 +9956,7 @@
       <c r="A215" s="11" t="n"/>
       <c r="B215" s="10" t="inlineStr">
         <is>
-          <t>PB5(CS111)-SRG,RJM/CL05</t>
+          <t>PB5,B6(CS111)-ASA,AM,SRG/CL10,11</t>
         </is>
       </c>
       <c r="C215" s="4" t="n"/>
@@ -10059,11 +9986,7 @@
     </row>
     <row r="216" ht="15.75" customHeight="1">
       <c r="A216" s="11" t="n"/>
-      <c r="B216" s="10" t="inlineStr">
-        <is>
-          <t>PB6(CS111)-ASA,AM/CL01</t>
-        </is>
-      </c>
+      <c r="B216" s="10" t="inlineStr"/>
       <c r="C216" s="4" t="n"/>
       <c r="D216" s="12" t="inlineStr"/>
       <c r="E216" s="12" t="inlineStr"/>
@@ -10091,7 +10014,7 @@
     </row>
     <row r="217" ht="15.75" customHeight="1">
       <c r="A217" s="11" t="n"/>
-      <c r="B217" s="24" t="inlineStr">
+      <c r="B217" s="10" t="inlineStr">
         <is>
           <t>PA17(EC111)-BEL1/VGO,CBP</t>
         </is>
@@ -10123,7 +10046,7 @@
     </row>
     <row r="218" ht="15.75" customHeight="1">
       <c r="A218" s="11" t="n"/>
-      <c r="B218" s="24" t="inlineStr">
+      <c r="B218" s="10" t="inlineStr">
         <is>
           <t>PA18(EC111)-BEL2/ALJ,VSS</t>
         </is>
@@ -10162,7 +10085,7 @@
       </c>
       <c r="C219" s="3" t="n"/>
       <c r="D219" s="4" t="n"/>
-      <c r="E219" s="17" t="inlineStr"/>
+      <c r="E219" s="16" t="inlineStr"/>
       <c r="F219" s="10" t="inlineStr"/>
       <c r="G219" s="10" t="inlineStr"/>
       <c r="H219" s="10" t="inlineStr"/>
@@ -10251,7 +10174,7 @@
     </row>
     <row r="222" ht="15.75" customHeight="1">
       <c r="A222" s="11" t="n"/>
-      <c r="B222" s="17" t="inlineStr"/>
+      <c r="B222" s="16" t="inlineStr"/>
       <c r="C222" s="10" t="inlineStr">
         <is>
           <t>PD4GE111)-CAD4/GRP</t>
@@ -10282,10 +10205,10 @@
       <c r="Z222" s="1" t="inlineStr"/>
     </row>
     <row r="223" ht="15.75" customHeight="1">
-      <c r="A223" s="19" t="n"/>
+      <c r="A223" s="17" t="n"/>
       <c r="B223" s="12" t="inlineStr"/>
       <c r="C223" s="12" t="inlineStr"/>
-      <c r="D223" s="17" t="inlineStr"/>
+      <c r="D223" s="16" t="inlineStr"/>
       <c r="E223" s="13" t="inlineStr"/>
       <c r="F223" s="10" t="inlineStr"/>
       <c r="G223" s="10" t="inlineStr"/>
@@ -10311,14 +10234,14 @@
     </row>
     <row r="224" ht="10.5" customHeight="1">
       <c r="A224" s="9" t="inlineStr"/>
-      <c r="B224" s="25" t="inlineStr"/>
-      <c r="C224" s="25" t="inlineStr"/>
-      <c r="D224" s="25" t="inlineStr"/>
-      <c r="E224" s="26" t="inlineStr"/>
-      <c r="F224" s="25" t="inlineStr"/>
-      <c r="G224" s="25" t="inlineStr"/>
-      <c r="H224" s="25" t="inlineStr"/>
-      <c r="I224" s="25" t="inlineStr"/>
+      <c r="B224" s="22" t="inlineStr"/>
+      <c r="C224" s="22" t="inlineStr"/>
+      <c r="D224" s="22" t="inlineStr"/>
+      <c r="E224" s="23" t="inlineStr"/>
+      <c r="F224" s="22" t="inlineStr"/>
+      <c r="G224" s="22" t="inlineStr"/>
+      <c r="H224" s="22" t="inlineStr"/>
+      <c r="I224" s="22" t="inlineStr"/>
       <c r="J224" s="5" t="inlineStr"/>
       <c r="K224" s="1" t="inlineStr"/>
       <c r="L224" s="1" t="inlineStr"/>
@@ -10370,15 +10293,15 @@
       <c r="Z225" s="1" t="inlineStr"/>
     </row>
     <row r="226" ht="5.25" customHeight="1">
-      <c r="A226" s="21" t="inlineStr"/>
-      <c r="B226" s="21" t="inlineStr"/>
-      <c r="C226" s="21" t="inlineStr"/>
-      <c r="D226" s="21" t="inlineStr"/>
-      <c r="E226" s="21" t="inlineStr"/>
-      <c r="F226" s="21" t="inlineStr"/>
-      <c r="G226" s="21" t="inlineStr"/>
-      <c r="H226" s="21" t="inlineStr"/>
-      <c r="I226" s="21" t="inlineStr"/>
+      <c r="A226" s="19" t="inlineStr"/>
+      <c r="B226" s="19" t="inlineStr"/>
+      <c r="C226" s="19" t="inlineStr"/>
+      <c r="D226" s="19" t="inlineStr"/>
+      <c r="E226" s="19" t="inlineStr"/>
+      <c r="F226" s="19" t="inlineStr"/>
+      <c r="G226" s="19" t="inlineStr"/>
+      <c r="H226" s="19" t="inlineStr"/>
+      <c r="I226" s="19" t="inlineStr"/>
       <c r="J226" s="5" t="inlineStr"/>
       <c r="K226" s="1" t="inlineStr"/>
       <c r="L226" s="1" t="inlineStr"/>
@@ -10430,7 +10353,7 @@
       <c r="Z227" s="1" t="inlineStr"/>
     </row>
     <row r="228" ht="18" customHeight="1">
-      <c r="A228" s="17" t="inlineStr"/>
+      <c r="A228" s="16" t="inlineStr"/>
       <c r="B228" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">A :  A1-A18 for students of ECE and Dual-ECE. Each section will consists of  batches of approximately 30 students. </t>
@@ -10462,7 +10385,7 @@
       <c r="Z228" s="1" t="inlineStr"/>
     </row>
     <row r="229" ht="18" customHeight="1">
-      <c r="A229" s="17" t="inlineStr"/>
+      <c r="A229" s="16" t="inlineStr"/>
       <c r="B229" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">B :  B1-B15 for students of CSE, IT and  Dual-CSE. Each section will consists of  batches of approximately 30 students. </t>
@@ -10494,7 +10417,7 @@
       <c r="Z229" s="1" t="inlineStr"/>
     </row>
     <row r="230" ht="18" customHeight="1">
-      <c r="A230" s="17" t="inlineStr"/>
+      <c r="A230" s="16" t="inlineStr"/>
       <c r="B230" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">C: C1-C3 for students of Bio Tech. Each section will consists of  batches of approximately 30 students. </t>
@@ -10526,7 +10449,7 @@
       <c r="Z230" s="1" t="inlineStr"/>
     </row>
     <row r="231" ht="18" customHeight="1">
-      <c r="A231" s="17" t="inlineStr"/>
+      <c r="A231" s="16" t="inlineStr"/>
       <c r="B231" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">G: G1-G4 for students of MNC. Each section will consists of  batches of approximately 30 students. </t>
@@ -10558,7 +10481,7 @@
       <c r="Z231" s="1" t="inlineStr"/>
     </row>
     <row r="232" ht="18" customHeight="1">
-      <c r="A232" s="17" t="inlineStr"/>
+      <c r="A232" s="16" t="inlineStr"/>
       <c r="B232" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">D: D1-D2 for students of Robotics &amp; AI. Each section will consists of  batches of approximately 30 students. </t>
@@ -10590,7 +10513,7 @@
       <c r="Z232" s="1" t="inlineStr"/>
     </row>
     <row r="233" ht="18" customHeight="1">
-      <c r="A233" s="17" t="inlineStr"/>
+      <c r="A233" s="16" t="inlineStr"/>
       <c r="B233" s="13" t="inlineStr">
         <is>
           <t>LT1, LT2 ….,G7,G8….,FF1,FF2….,F1, F3, are lecture theatres, TS1,TS2…….are tutorial rooms &amp; CS1,CS2.. are classrooms.</t>
@@ -10655,7 +10578,7 @@
     </row>
     <row r="235" ht="18" customHeight="1">
       <c r="A235" s="10" t="inlineStr"/>
-      <c r="B235" s="17" t="inlineStr">
+      <c r="B235" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">Example:  </t>
         </is>
@@ -10665,7 +10588,7 @@
           <t>LC1,C2,C3(PH112)-G7/AP</t>
         </is>
       </c>
-      <c r="D235" s="27" t="inlineStr">
+      <c r="D235" s="24" t="inlineStr">
         <is>
           <t>means lecture class of C1, C2,C3  of the  course PH112  in the room (G2)- to be taught by faculty Prof. Anirban Pathak (AP).</t>
         </is>
@@ -10695,13 +10618,13 @@
     </row>
     <row r="236" ht="18" customHeight="1">
       <c r="A236" s="11" t="n"/>
-      <c r="B236" s="17" t="inlineStr"/>
+      <c r="B236" s="16" t="inlineStr"/>
       <c r="C236" s="13" t="inlineStr">
         <is>
           <t>TG1(MA111)--/PAT</t>
         </is>
       </c>
-      <c r="D236" s="27" t="inlineStr">
+      <c r="D236" s="24" t="inlineStr">
         <is>
           <t>means tutorial class of subsection G1 of the course MAT111 in tutorial room (-)- to be taught by faculty Prof. Pato Kumari (PAT).</t>
         </is>
@@ -10730,14 +10653,14 @@
       <c r="Z236" s="1" t="inlineStr"/>
     </row>
     <row r="237" ht="18" customHeight="1">
-      <c r="A237" s="19" t="n"/>
-      <c r="B237" s="17" t="inlineStr"/>
+      <c r="A237" s="17" t="n"/>
+      <c r="B237" s="16" t="inlineStr"/>
       <c r="C237" s="10" t="inlineStr">
         <is>
           <t>PD1(PH171)-PL1/NAR</t>
         </is>
       </c>
-      <c r="D237" s="27" t="inlineStr">
+      <c r="D237" s="24" t="inlineStr">
         <is>
           <t>means practical class of subsection D1 of the course PH171  in Physics Laboratory1 (PL1)-to be taught by faculty Dr. Narinder Kaur (NAR).</t>
         </is>
@@ -10767,9 +10690,9 @@
     </row>
     <row r="238" ht="6" customHeight="1">
       <c r="A238" s="1" t="inlineStr"/>
-      <c r="B238" s="17" t="inlineStr"/>
+      <c r="B238" s="16" t="inlineStr"/>
       <c r="C238" s="10" t="inlineStr"/>
-      <c r="D238" s="27" t="inlineStr"/>
+      <c r="D238" s="24" t="inlineStr"/>
       <c r="E238" s="1" t="inlineStr"/>
       <c r="F238" s="1" t="inlineStr"/>
       <c r="G238" s="1" t="inlineStr"/>
@@ -10795,42 +10718,42 @@
     </row>
     <row r="239" ht="27.75" customHeight="1">
       <c r="A239" s="10" t="inlineStr"/>
-      <c r="B239" s="28" t="inlineStr">
+      <c r="B239" s="25" t="inlineStr">
         <is>
           <t>Faculty Abbreviation with Names</t>
         </is>
       </c>
-      <c r="C239" s="29" t="inlineStr">
+      <c r="C239" s="26" t="inlineStr">
         <is>
           <t>Faculty Abbreviation with Names</t>
         </is>
       </c>
-      <c r="D239" s="28" t="inlineStr">
+      <c r="D239" s="25" t="inlineStr">
         <is>
           <t>Faculty Abbreviation with Names</t>
         </is>
       </c>
-      <c r="E239" s="28" t="inlineStr">
+      <c r="E239" s="25" t="inlineStr">
         <is>
           <t>Faculty Abbreviation with Names</t>
         </is>
       </c>
-      <c r="F239" s="28" t="inlineStr">
+      <c r="F239" s="25" t="inlineStr">
         <is>
           <t>Faculty Abbreviation with Names</t>
         </is>
       </c>
-      <c r="G239" s="28" t="inlineStr">
+      <c r="G239" s="25" t="inlineStr">
         <is>
           <t>Faculty Abbreviation with Names</t>
         </is>
       </c>
-      <c r="H239" s="28" t="inlineStr">
+      <c r="H239" s="25" t="inlineStr">
         <is>
           <t>SHORT FORM / SUBJECT CODE</t>
         </is>
       </c>
-      <c r="I239" s="28" t="inlineStr">
+      <c r="I239" s="25" t="inlineStr">
         <is>
           <t>SUBJECT NAME</t>
         </is>
@@ -10855,42 +10778,42 @@
     </row>
     <row r="240" ht="15.75" customHeight="1">
       <c r="A240" s="11" t="n"/>
-      <c r="B240" s="30" t="inlineStr">
+      <c r="B240" s="27" t="inlineStr">
         <is>
           <t>AB: Ankur Bhardwaj</t>
         </is>
       </c>
-      <c r="C240" s="30" t="inlineStr">
+      <c r="C240" s="27" t="inlineStr">
         <is>
           <t>BB: BADRI BAJAJ</t>
         </is>
       </c>
-      <c r="D240" s="30" t="inlineStr">
+      <c r="D240" s="27" t="inlineStr">
         <is>
           <t>HPT: Dr. Himani Pant</t>
         </is>
       </c>
-      <c r="E240" s="30" t="inlineStr">
+      <c r="E240" s="27" t="inlineStr">
         <is>
           <t>NAC: NAVEEN CHAUHAN</t>
         </is>
       </c>
-      <c r="F240" s="30" t="inlineStr">
+      <c r="F240" s="27" t="inlineStr">
         <is>
           <t>RCA: RICHA KUSHWAHA</t>
         </is>
       </c>
-      <c r="G240" s="30" t="inlineStr">
+      <c r="G240" s="27" t="inlineStr">
         <is>
           <t>SIM: Simmi Sharma</t>
         </is>
       </c>
-      <c r="H240" s="31" t="inlineStr">
+      <c r="H240" s="28" t="inlineStr">
         <is>
           <t>HS112/15B11HS112</t>
         </is>
       </c>
-      <c r="I240" s="32" t="inlineStr">
+      <c r="I240" s="29" t="inlineStr">
         <is>
           <t>English</t>
         </is>
@@ -10915,43 +10838,43 @@
     </row>
     <row r="241" ht="31.5" customHeight="1">
       <c r="A241" s="11" t="n"/>
-      <c r="B241" s="33" t="inlineStr">
+      <c r="B241" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">ABH: Dr. Ashish Batnagar 
 </t>
         </is>
       </c>
-      <c r="C241" s="30" t="inlineStr">
+      <c r="C241" s="27" t="inlineStr">
         <is>
           <t>BCJ: Dr. Bhubesh Chander Joshi</t>
         </is>
       </c>
-      <c r="D241" s="30" t="inlineStr">
+      <c r="D241" s="27" t="inlineStr">
         <is>
           <t>INC: Dr. Indrani Chakarborty</t>
         </is>
       </c>
-      <c r="E241" s="30" t="inlineStr">
+      <c r="E241" s="27" t="inlineStr">
         <is>
           <t>NAR: Dr. Narinder Kaur</t>
         </is>
       </c>
-      <c r="F241" s="30" t="inlineStr">
+      <c r="F241" s="27" t="inlineStr">
         <is>
           <t>RHA: Rachna Singh</t>
         </is>
       </c>
-      <c r="G241" s="30" t="inlineStr">
+      <c r="G241" s="27" t="inlineStr">
         <is>
           <t>SLK: SILKI KHARALIYA</t>
         </is>
       </c>
-      <c r="H241" s="31" t="inlineStr">
+      <c r="H241" s="28" t="inlineStr">
         <is>
           <t>CI111/15B11CI111</t>
         </is>
       </c>
-      <c r="I241" s="34" t="inlineStr">
+      <c r="I241" s="31" t="inlineStr">
         <is>
           <t>Software Development Fundamentals- I</t>
         </is>
@@ -10976,42 +10899,42 @@
     </row>
     <row r="242" ht="30.75" customHeight="1">
       <c r="A242" s="11" t="n"/>
-      <c r="B242" s="30" t="inlineStr">
+      <c r="B242" s="27" t="inlineStr">
         <is>
           <t>ABU: Abhijeet Upadhyay</t>
         </is>
       </c>
-      <c r="C242" s="30" t="inlineStr">
+      <c r="C242" s="27" t="inlineStr">
         <is>
           <t>BHA: Bhawna Gupta</t>
         </is>
       </c>
-      <c r="D242" s="30" t="inlineStr">
+      <c r="D242" s="27" t="inlineStr">
         <is>
           <t>JG: Juhi gupta</t>
         </is>
       </c>
-      <c r="E242" s="30" t="inlineStr">
+      <c r="E242" s="27" t="inlineStr">
         <is>
           <t>NBH: Neha Bhadauria</t>
         </is>
       </c>
-      <c r="F242" s="30" t="inlineStr">
+      <c r="F242" s="27" t="inlineStr">
         <is>
           <t>RJM: RAJIV KUMAR MISHRA</t>
         </is>
       </c>
-      <c r="G242" s="30" t="inlineStr">
+      <c r="G242" s="27" t="inlineStr">
         <is>
           <t>SLM: Salman Khan</t>
         </is>
       </c>
-      <c r="H242" s="30" t="inlineStr">
+      <c r="H242" s="27" t="inlineStr">
         <is>
           <t>CS111/24B15CS111</t>
         </is>
       </c>
-      <c r="I242" s="35" t="inlineStr">
+      <c r="I242" s="32" t="inlineStr">
         <is>
           <t>Software Development Fundamentals- I Lab</t>
         </is>
@@ -11036,42 +10959,42 @@
     </row>
     <row r="243" ht="30" customHeight="1">
       <c r="A243" s="11" t="n"/>
-      <c r="B243" s="30" t="inlineStr">
+      <c r="B243" s="27" t="inlineStr">
         <is>
           <t>ADM: Adhirath Mandal</t>
         </is>
       </c>
-      <c r="C243" s="30" t="inlineStr">
+      <c r="C243" s="27" t="inlineStr">
         <is>
           <t>BVI: Bhuvneshwari S</t>
         </is>
       </c>
-      <c r="D243" s="30" t="inlineStr">
+      <c r="D243" s="27" t="inlineStr">
         <is>
           <t>JMO: Jitendra Mohan</t>
         </is>
       </c>
-      <c r="E243" s="30" t="inlineStr">
+      <c r="E243" s="27" t="inlineStr">
         <is>
           <t>NEJ: Neetu Joshi</t>
         </is>
       </c>
-      <c r="F243" s="30" t="inlineStr">
+      <c r="F243" s="27" t="inlineStr">
         <is>
           <t>RKD: Prof. Rakesh Kumar Dwivedi</t>
         </is>
       </c>
-      <c r="G243" s="30" t="inlineStr">
+      <c r="G243" s="27" t="inlineStr">
         <is>
           <t>SMK: Samriti Kalia</t>
         </is>
       </c>
-      <c r="H243" s="30" t="inlineStr">
+      <c r="H243" s="27" t="inlineStr">
         <is>
           <t>18CI111/18B11CI111</t>
         </is>
       </c>
-      <c r="I243" s="35" t="inlineStr">
+      <c r="I243" s="32" t="inlineStr">
         <is>
           <t>Fundamentals of Computers &amp; Programming - I</t>
         </is>
@@ -11096,42 +11019,42 @@
     </row>
     <row r="244" ht="30" customHeight="1">
       <c r="A244" s="11" t="n"/>
-      <c r="B244" s="30" t="inlineStr">
+      <c r="B244" s="27" t="inlineStr">
         <is>
           <t>AJS: ANKITA JAISWAL</t>
         </is>
       </c>
-      <c r="C244" s="30" t="inlineStr">
+      <c r="C244" s="27" t="inlineStr">
         <is>
           <t>CDN: Chandan Kumar</t>
         </is>
       </c>
-      <c r="D244" s="30" t="inlineStr">
+      <c r="D244" s="27" t="inlineStr">
         <is>
           <t>JYM: Jyoti Mishra</t>
         </is>
       </c>
-      <c r="E244" s="30" t="inlineStr">
+      <c r="E244" s="27" t="inlineStr">
         <is>
           <t>NG: Dr. Navendu Goswami</t>
         </is>
       </c>
-      <c r="F244" s="30" t="inlineStr">
+      <c r="F244" s="27" t="inlineStr">
         <is>
           <t>RKG: Dr. Radha Krishan Gopal</t>
         </is>
       </c>
-      <c r="G244" s="30" t="inlineStr">
+      <c r="G244" s="27" t="inlineStr">
         <is>
           <t>SMS: SUMESHWAR SINGH</t>
         </is>
       </c>
-      <c r="H244" s="36" t="inlineStr">
+      <c r="H244" s="27" t="inlineStr">
         <is>
           <t>24CS111/24B45CS111</t>
         </is>
       </c>
-      <c r="I244" s="35" t="inlineStr">
+      <c r="I244" s="32" t="inlineStr">
         <is>
           <t>Fundamentals of Computers &amp; Programming - I Lab</t>
         </is>
@@ -11156,42 +11079,42 @@
     </row>
     <row r="245" ht="15" customHeight="1">
       <c r="A245" s="11" t="n"/>
-      <c r="B245" s="30" t="inlineStr">
+      <c r="B245" s="27" t="inlineStr">
         <is>
           <t>AKT: AKSHIT RAJ PATEL</t>
         </is>
       </c>
-      <c r="C245" s="30" t="inlineStr">
+      <c r="C245" s="27" t="inlineStr">
         <is>
           <t>DAM: Dr. Damanpreet Kaur</t>
         </is>
       </c>
-      <c r="D245" s="30" t="inlineStr">
+      <c r="D245" s="27" t="inlineStr">
         <is>
           <t>KMB: KANUPRIYA MISRA BAKHRU</t>
         </is>
       </c>
-      <c r="E245" s="30" t="inlineStr">
+      <c r="E245" s="27" t="inlineStr">
         <is>
           <t>NHI: Nidhi Tewari</t>
         </is>
       </c>
-      <c r="F245" s="30" t="inlineStr">
+      <c r="F245" s="27" t="inlineStr">
         <is>
           <t>ROH: ROHIT KUMAR SONY</t>
         </is>
       </c>
-      <c r="G245" s="30" t="inlineStr">
+      <c r="G245" s="27" t="inlineStr">
         <is>
           <t>SND: Dr. Sandeep Mishra</t>
         </is>
       </c>
-      <c r="H245" s="30" t="inlineStr">
+      <c r="H245" s="27" t="inlineStr">
         <is>
           <t>EC111/ 24B11EC111</t>
         </is>
       </c>
-      <c r="I245" s="35" t="inlineStr">
+      <c r="I245" s="32" t="inlineStr">
         <is>
           <t>Basic Electronics</t>
         </is>
@@ -11216,42 +11139,42 @@
     </row>
     <row r="246" ht="15" customHeight="1">
       <c r="A246" s="11" t="n"/>
-      <c r="B246" s="30" t="inlineStr">
+      <c r="B246" s="27" t="inlineStr">
         <is>
           <t>ALJ: Alok Joshi</t>
         </is>
       </c>
-      <c r="C246" s="30" t="inlineStr">
+      <c r="C246" s="27" t="inlineStr">
         <is>
           <t>DCH: DIKSHA CHAWLA</t>
         </is>
       </c>
-      <c r="D246" s="30" t="inlineStr">
+      <c r="D246" s="27" t="inlineStr">
         <is>
           <t>KNP: KANU PRIYA</t>
         </is>
       </c>
-      <c r="E246" s="30" t="inlineStr">
+      <c r="E246" s="27" t="inlineStr">
         <is>
           <t>NIS: NIBHA SINHA</t>
         </is>
       </c>
-      <c r="F246" s="30" t="inlineStr">
+      <c r="F246" s="27" t="inlineStr">
         <is>
           <t>RRJ: Rituraj</t>
         </is>
       </c>
-      <c r="G246" s="30" t="inlineStr">
+      <c r="G246" s="27" t="inlineStr">
         <is>
           <t>SNP: SatyaNarayan Patel</t>
         </is>
       </c>
-      <c r="H246" s="30" t="inlineStr">
+      <c r="H246" s="27" t="inlineStr">
         <is>
           <t>EC111 / 24B15EC111</t>
         </is>
       </c>
-      <c r="I246" s="35" t="inlineStr">
+      <c r="I246" s="32" t="inlineStr">
         <is>
           <t>Basic Electronics Lab</t>
         </is>
@@ -11276,42 +11199,42 @@
     </row>
     <row r="247" ht="15" customHeight="1">
       <c r="A247" s="11" t="n"/>
-      <c r="B247" s="30" t="inlineStr">
+      <c r="B247" s="27" t="inlineStr">
         <is>
           <t>AM: ASHISH MISHRA</t>
         </is>
       </c>
-      <c r="C247" s="30" t="inlineStr">
+      <c r="C247" s="27" t="inlineStr">
         <is>
           <t>DCS:Dr Dinesh Bisht</t>
         </is>
       </c>
-      <c r="D247" s="30" t="inlineStr">
+      <c r="D247" s="27" t="inlineStr">
         <is>
           <t>KUL: Kuldeep Baderia</t>
         </is>
       </c>
-      <c r="E247" s="30" t="inlineStr">
+      <c r="E247" s="27" t="inlineStr">
         <is>
           <t>NIY: NIYATI AGGRAWAL</t>
         </is>
       </c>
-      <c r="F247" s="30" t="inlineStr">
+      <c r="F247" s="27" t="inlineStr">
         <is>
           <t>RRP: Radha Raman Pandey</t>
         </is>
       </c>
-      <c r="G247" s="30" t="inlineStr">
+      <c r="G247" s="27" t="inlineStr">
         <is>
           <t>SOS: SONAL SAURABH</t>
         </is>
       </c>
-      <c r="H247" s="30" t="inlineStr">
+      <c r="H247" s="27" t="inlineStr">
         <is>
           <t>EC112/ 24B11EC112</t>
         </is>
       </c>
-      <c r="I247" s="35" t="inlineStr">
+      <c r="I247" s="32" t="inlineStr">
         <is>
           <t>Basic Electronics</t>
         </is>
@@ -11336,42 +11259,42 @@
     </row>
     <row r="248" ht="15" customHeight="1">
       <c r="A248" s="11" t="n"/>
-      <c r="B248" s="30" t="inlineStr">
+      <c r="B248" s="27" t="inlineStr">
         <is>
           <t>AMI: ANKITA MISHRA</t>
         </is>
       </c>
-      <c r="C248" s="30" t="inlineStr">
+      <c r="C248" s="27" t="inlineStr">
         <is>
           <t>DGA:Dr. Diksha Gupta</t>
         </is>
       </c>
-      <c r="D248" s="30" t="inlineStr">
+      <c r="D248" s="27" t="inlineStr">
         <is>
           <t>LK: Prof. Lokendra Kumar</t>
         </is>
       </c>
-      <c r="E248" s="30" t="inlineStr">
+      <c r="E248" s="27" t="inlineStr">
         <is>
           <t>NKS: Dr. Navneet K. Sharma</t>
         </is>
       </c>
-      <c r="F248" s="30" t="inlineStr">
+      <c r="F248" s="27" t="inlineStr">
         <is>
           <t>RS: Ritesh Sharma</t>
         </is>
       </c>
-      <c r="G248" s="30" t="inlineStr">
+      <c r="G248" s="27" t="inlineStr">
         <is>
           <t>SP:Dr. Shikha Pandey</t>
         </is>
       </c>
-      <c r="H248" s="30" t="inlineStr">
+      <c r="H248" s="27" t="inlineStr">
         <is>
           <t>EC112 / 24B15EC112</t>
         </is>
       </c>
-      <c r="I248" s="35" t="inlineStr">
+      <c r="I248" s="32" t="inlineStr">
         <is>
           <t>Basic Electronics Lab</t>
         </is>
@@ -11396,42 +11319,42 @@
     </row>
     <row r="249" ht="15" customHeight="1">
       <c r="A249" s="11" t="n"/>
-      <c r="B249" s="30" t="inlineStr">
+      <c r="B249" s="27" t="inlineStr">
         <is>
           <t>AN: Dr. Anuj Bhardwa</t>
         </is>
       </c>
-      <c r="C249" s="30" t="inlineStr">
+      <c r="C249" s="27" t="inlineStr">
         <is>
           <t>DIN: Dr. Dinesh Tripathi</t>
         </is>
       </c>
-      <c r="D249" s="30" t="inlineStr">
+      <c r="D249" s="27" t="inlineStr">
         <is>
           <t>MAY: MAYURI GUPTA</t>
         </is>
       </c>
-      <c r="E249" s="30" t="inlineStr">
+      <c r="E249" s="27" t="inlineStr">
         <is>
           <t>NS:Dr. Neha Singhal</t>
         </is>
       </c>
-      <c r="F249" s="30" t="inlineStr">
+      <c r="F249" s="27" t="inlineStr">
         <is>
           <t>RSA:Dr. Rupali Srivastav</t>
         </is>
       </c>
-      <c r="G249" s="30" t="inlineStr">
+      <c r="G249" s="27" t="inlineStr">
         <is>
           <t>SPP: Prof. S.P. Purohit</t>
         </is>
       </c>
-      <c r="H249" s="30" t="inlineStr">
+      <c r="H249" s="27" t="inlineStr">
         <is>
           <t>GE111/18B15GE111</t>
         </is>
       </c>
-      <c r="I249" s="35" t="inlineStr">
+      <c r="I249" s="32" t="inlineStr">
         <is>
           <t>Engineering Drawing and Design</t>
         </is>
@@ -11456,42 +11379,42 @@
     </row>
     <row r="250" ht="15" customHeight="1">
       <c r="A250" s="11" t="n"/>
-      <c r="B250" s="30" t="inlineStr">
+      <c r="B250" s="27" t="inlineStr">
         <is>
           <t>ANP: ANUPAMA PADHA</t>
         </is>
       </c>
-      <c r="C250" s="30" t="inlineStr">
+      <c r="C250" s="27" t="inlineStr">
         <is>
           <t>DIP: Dr. Dipiti Yadav</t>
         </is>
       </c>
-      <c r="D250" s="30" t="inlineStr">
+      <c r="D250" s="27" t="inlineStr">
         <is>
           <t>MB:MONALI BHATTACHARYA</t>
         </is>
       </c>
-      <c r="E250" s="30" t="inlineStr">
+      <c r="E250" s="27" t="inlineStr">
         <is>
           <t>NSH: K.Nisha</t>
         </is>
       </c>
-      <c r="F250" s="30" t="inlineStr">
+      <c r="F250" s="27" t="inlineStr">
         <is>
           <t>RSC: Dr. RAM SURAT CHAUHAN</t>
         </is>
       </c>
-      <c r="G250" s="30" t="inlineStr">
+      <c r="G250" s="27" t="inlineStr">
         <is>
           <t>SRG: SARISHTY GUPTA</t>
         </is>
       </c>
-      <c r="H250" s="30" t="inlineStr">
+      <c r="H250" s="27" t="inlineStr">
         <is>
           <t>PH111 / 15B11PH111</t>
         </is>
       </c>
-      <c r="I250" s="35" t="inlineStr">
+      <c r="I250" s="32" t="inlineStr">
         <is>
           <t>Physics-1</t>
         </is>
@@ -11516,42 +11439,42 @@
     </row>
     <row r="251" ht="15" customHeight="1">
       <c r="A251" s="11" t="n"/>
-      <c r="B251" s="30" t="inlineStr">
+      <c r="B251" s="27" t="inlineStr">
         <is>
           <t>ANU: Dr. Anuraj Panwar</t>
         </is>
       </c>
-      <c r="C251" s="30" t="inlineStr">
+      <c r="C251" s="27" t="inlineStr">
         <is>
           <t>DSI: DEEPTI</t>
         </is>
       </c>
-      <c r="D251" s="30" t="inlineStr">
+      <c r="D251" s="27" t="inlineStr">
         <is>
           <t>MDU: MOHUA DUTTA</t>
         </is>
       </c>
-      <c r="E251" s="30" t="inlineStr">
+      <c r="E251" s="27" t="inlineStr">
         <is>
           <t>NSK:Dr. Nisha Shukla</t>
         </is>
       </c>
-      <c r="F251" s="30" t="inlineStr">
+      <c r="F251" s="27" t="inlineStr">
         <is>
           <t>RSH:Dr. Richa Sharma</t>
         </is>
       </c>
-      <c r="G251" s="30" t="inlineStr">
+      <c r="G251" s="27" t="inlineStr">
         <is>
           <t>SWET: Shwetabh Singh</t>
         </is>
       </c>
-      <c r="H251" s="30" t="inlineStr">
+      <c r="H251" s="27" t="inlineStr">
         <is>
           <t>PH112 / 15B11PH112</t>
         </is>
       </c>
-      <c r="I251" s="35" t="inlineStr">
+      <c r="I251" s="32" t="inlineStr">
         <is>
           <t>Physics for Biotechnology</t>
         </is>
@@ -11576,42 +11499,42 @@
     </row>
     <row r="252" ht="15" customHeight="1">
       <c r="A252" s="11" t="n"/>
-      <c r="B252" s="30" t="inlineStr">
+      <c r="B252" s="27" t="inlineStr">
         <is>
           <t>ANV: ANKIT VIDYARTHI</t>
         </is>
       </c>
-      <c r="C252" s="30" t="inlineStr">
+      <c r="C252" s="27" t="inlineStr">
         <is>
           <t>EKS: EKTA SINGH</t>
         </is>
       </c>
-      <c r="D252" s="30" t="inlineStr">
+      <c r="D252" s="27" t="inlineStr">
         <is>
           <t>MGR: MEGHA RATHI</t>
         </is>
       </c>
-      <c r="E252" s="30" t="inlineStr">
+      <c r="E252" s="27" t="inlineStr">
         <is>
           <t>NTN: Nitin Muchal</t>
         </is>
       </c>
-      <c r="F252" s="30" t="inlineStr">
+      <c r="F252" s="27" t="inlineStr">
         <is>
           <t>RU: Ruby Beniwal</t>
         </is>
       </c>
-      <c r="G252" s="30" t="inlineStr">
+      <c r="G252" s="27" t="inlineStr">
         <is>
           <t>TAJ: TAJ ALAM</t>
         </is>
       </c>
-      <c r="H252" s="30" t="inlineStr">
+      <c r="H252" s="27" t="inlineStr">
         <is>
           <t>PH171 / 15B17PH171</t>
         </is>
       </c>
-      <c r="I252" s="35" t="inlineStr">
+      <c r="I252" s="32" t="inlineStr">
         <is>
           <t>Physics Lab-1</t>
         </is>
@@ -11636,38 +11559,38 @@
     </row>
     <row r="253" ht="15" customHeight="1">
       <c r="A253" s="11" t="n"/>
-      <c r="B253" s="30" t="inlineStr">
+      <c r="B253" s="27" t="inlineStr">
         <is>
           <t>AP: Prof. Anirban Pathak</t>
         </is>
       </c>
-      <c r="C253" s="30" t="inlineStr">
+      <c r="C253" s="27" t="inlineStr">
         <is>
           <t>EKY: Dr. Ekta Yadav</t>
         </is>
       </c>
-      <c r="D253" s="30" t="inlineStr">
+      <c r="D253" s="27" t="inlineStr">
         <is>
           <t>MJ: Madhu Jain</t>
         </is>
       </c>
-      <c r="E253" s="30" t="inlineStr">
+      <c r="E253" s="27" t="inlineStr">
         <is>
           <t>NTS: Nitesh Singh</t>
         </is>
       </c>
-      <c r="F253" s="30" t="inlineStr">
+      <c r="F253" s="27" t="inlineStr">
         <is>
           <t>SAA: SAKSHI GUPTA</t>
         </is>
       </c>
-      <c r="G253" s="30" t="inlineStr">
+      <c r="G253" s="27" t="inlineStr">
         <is>
           <t>TNV: TANVI GAUTAM</t>
         </is>
       </c>
-      <c r="H253" s="32" t="inlineStr"/>
-      <c r="I253" s="37" t="inlineStr"/>
+      <c r="H253" s="29" t="inlineStr"/>
+      <c r="I253" s="33" t="inlineStr"/>
       <c r="J253" s="5" t="inlineStr"/>
       <c r="K253" s="1" t="inlineStr"/>
       <c r="L253" s="1" t="inlineStr"/>
@@ -11688,38 +11611,38 @@
     </row>
     <row r="254" ht="15" customHeight="1">
       <c r="A254" s="11" t="n"/>
-      <c r="B254" s="30" t="inlineStr">
+      <c r="B254" s="27" t="inlineStr">
         <is>
           <t>APR: AMANPREET KAUR</t>
         </is>
       </c>
-      <c r="C254" s="30" t="inlineStr">
+      <c r="C254" s="27" t="inlineStr">
         <is>
           <t>GA: Dr. Gaurav Aggrawal</t>
         </is>
       </c>
-      <c r="D254" s="30" t="inlineStr">
+      <c r="D254" s="27" t="inlineStr">
         <is>
           <t>MJH: Madhu Jhariya</t>
         </is>
       </c>
-      <c r="E254" s="30" t="inlineStr">
+      <c r="E254" s="27" t="inlineStr">
         <is>
           <t>PAC: PARIDHI</t>
         </is>
       </c>
-      <c r="F254" s="30" t="inlineStr">
+      <c r="F254" s="27" t="inlineStr">
         <is>
           <t>SDA: SURAJ DAS</t>
         </is>
       </c>
-      <c r="G254" s="30" t="inlineStr">
+      <c r="G254" s="27" t="inlineStr">
         <is>
           <t>VD: Vivek Dwivedi</t>
         </is>
       </c>
-      <c r="H254" s="32" t="inlineStr"/>
-      <c r="I254" s="37" t="inlineStr"/>
+      <c r="H254" s="29" t="inlineStr"/>
+      <c r="I254" s="33" t="inlineStr"/>
       <c r="J254" s="5" t="inlineStr"/>
       <c r="K254" s="1" t="inlineStr"/>
       <c r="L254" s="1" t="inlineStr"/>
@@ -11740,38 +11663,38 @@
     </row>
     <row r="255" ht="15" customHeight="1">
       <c r="A255" s="11" t="n"/>
-      <c r="B255" s="30" t="inlineStr">
+      <c r="B255" s="27" t="inlineStr">
         <is>
           <t>ASA: ANITA SAHOO</t>
         </is>
       </c>
-      <c r="C255" s="30" t="inlineStr">
+      <c r="C255" s="27" t="inlineStr">
         <is>
           <t>GGL: Gorav Gugliani</t>
         </is>
       </c>
-      <c r="D255" s="30" t="inlineStr">
+      <c r="D255" s="27" t="inlineStr">
         <is>
           <t>MKB:Dr. Manish Kumar Bansal</t>
         </is>
       </c>
-      <c r="E255" s="30" t="inlineStr">
+      <c r="E255" s="27" t="inlineStr">
         <is>
           <t>PC: Dr. Papia Chowdhury</t>
         </is>
       </c>
-      <c r="F255" s="30" t="inlineStr">
+      <c r="F255" s="27" t="inlineStr">
         <is>
           <t>SDC: Dr. Sandeep Chokker</t>
         </is>
       </c>
-      <c r="G255" s="30" t="inlineStr">
+      <c r="G255" s="27" t="inlineStr">
         <is>
           <t>VGO: Varun Goel</t>
         </is>
       </c>
-      <c r="H255" s="32" t="inlineStr"/>
-      <c r="I255" s="37" t="inlineStr"/>
+      <c r="H255" s="29" t="inlineStr"/>
+      <c r="I255" s="33" t="inlineStr"/>
       <c r="J255" s="5" t="inlineStr"/>
       <c r="K255" s="1" t="inlineStr"/>
       <c r="L255" s="1" t="inlineStr"/>
@@ -11792,39 +11715,39 @@
     </row>
     <row r="256" ht="15" customHeight="1">
       <c r="A256" s="11" t="n"/>
-      <c r="B256" s="30" t="inlineStr">
+      <c r="B256" s="27" t="inlineStr">
         <is>
           <t>ASG: Ashish Gupta</t>
         </is>
       </c>
-      <c r="C256" s="33" t="inlineStr">
+      <c r="C256" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">GPK: Dr. Guru Prasad Kadam 
 </t>
         </is>
       </c>
-      <c r="D256" s="30" t="inlineStr">
+      <c r="D256" s="27" t="inlineStr">
         <is>
           <t>MKC: Dr.Manoj Kumar</t>
         </is>
       </c>
-      <c r="E256" s="30" t="inlineStr">
+      <c r="E256" s="27" t="inlineStr">
         <is>
           <t>PKU: PRASHANT KAUSHIK</t>
         </is>
       </c>
-      <c r="F256" s="30" t="inlineStr">
+      <c r="F256" s="27" t="inlineStr">
         <is>
           <t>SGL:Dr. Shashank Goel</t>
         </is>
       </c>
-      <c r="G256" s="30" t="inlineStr">
+      <c r="G256" s="27" t="inlineStr">
         <is>
           <t>VKH: Vijay Khare</t>
         </is>
       </c>
-      <c r="H256" s="32" t="inlineStr"/>
-      <c r="I256" s="37" t="inlineStr"/>
+      <c r="H256" s="29" t="inlineStr"/>
+      <c r="I256" s="33" t="inlineStr"/>
       <c r="J256" s="5" t="inlineStr"/>
       <c r="K256" s="1" t="inlineStr"/>
       <c r="L256" s="1" t="inlineStr"/>
@@ -11845,38 +11768,38 @@
     </row>
     <row r="257" ht="15" customHeight="1">
       <c r="A257" s="11" t="n"/>
-      <c r="B257" s="30" t="inlineStr">
+      <c r="B257" s="27" t="inlineStr">
         <is>
           <t>ASU: ASHU KUMARI</t>
         </is>
       </c>
-      <c r="C257" s="30" t="inlineStr">
+      <c r="C257" s="27" t="inlineStr">
         <is>
           <t>GRP: Gaurav Patel</t>
         </is>
       </c>
-      <c r="D257" s="30" t="inlineStr">
+      <c r="D257" s="27" t="inlineStr">
         <is>
           <t>MKT: MANISH KUMAR THAKUR</t>
         </is>
       </c>
-      <c r="E257" s="30" t="inlineStr">
+      <c r="E257" s="27" t="inlineStr">
         <is>
           <t>PKY: Pankaj Yadav</t>
         </is>
       </c>
-      <c r="F257" s="30" t="inlineStr">
+      <c r="F257" s="27" t="inlineStr">
         <is>
           <t>SHA: Shamim Akhter</t>
         </is>
       </c>
-      <c r="G257" s="30" t="inlineStr">
+      <c r="G257" s="27" t="inlineStr">
         <is>
           <t>VRT: Dr. Vaibhav Rawoot</t>
         </is>
       </c>
-      <c r="H257" s="32" t="inlineStr"/>
-      <c r="I257" s="37" t="inlineStr"/>
+      <c r="H257" s="29" t="inlineStr"/>
+      <c r="I257" s="33" t="inlineStr"/>
       <c r="J257" s="5" t="inlineStr"/>
       <c r="K257" s="1" t="inlineStr"/>
       <c r="L257" s="1" t="inlineStr"/>
@@ -11897,35 +11820,35 @@
     </row>
     <row r="258" ht="15" customHeight="1">
       <c r="A258" s="11" t="n"/>
-      <c r="B258" s="30" t="inlineStr">
+      <c r="B258" s="27" t="inlineStr">
         <is>
           <t>ATA: Astha Sharma</t>
         </is>
       </c>
-      <c r="C258" s="30" t="inlineStr">
+      <c r="C258" s="27" t="inlineStr">
         <is>
           <t>GV: Gaurav Verma</t>
         </is>
       </c>
-      <c r="D258" s="30" t="inlineStr">
+      <c r="D258" s="27" t="inlineStr">
         <is>
           <t>MN: Mandeep Narula</t>
         </is>
       </c>
-      <c r="E258" s="30" t="inlineStr">
+      <c r="E258" s="27" t="inlineStr">
         <is>
           <t>PSI:Dr. Priya Shahi</t>
         </is>
       </c>
-      <c r="F258" s="33" t="inlineStr">
+      <c r="F258" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">SHIV: Dr. Shivani Singh 
 </t>
         </is>
       </c>
-      <c r="G258" s="30" t="inlineStr"/>
-      <c r="H258" s="32" t="inlineStr"/>
-      <c r="I258" s="37" t="inlineStr"/>
+      <c r="G258" s="27" t="inlineStr"/>
+      <c r="H258" s="29" t="inlineStr"/>
+      <c r="I258" s="33" t="inlineStr"/>
       <c r="J258" s="5" t="inlineStr"/>
       <c r="K258" s="1" t="inlineStr"/>
       <c r="L258" s="1" t="inlineStr"/>
@@ -11946,34 +11869,34 @@
     </row>
     <row r="259" ht="15" customHeight="1">
       <c r="A259" s="11" t="n"/>
-      <c r="B259" s="30" t="inlineStr">
+      <c r="B259" s="27" t="inlineStr">
         <is>
           <t>AVR: ANKITA VERMA</t>
         </is>
       </c>
-      <c r="C259" s="30" t="inlineStr">
+      <c r="C259" s="27" t="inlineStr">
         <is>
           <t>HA:Dr. Himanshu Agarwal</t>
         </is>
       </c>
-      <c r="D259" s="30" t="inlineStr">
+      <c r="D259" s="27" t="inlineStr">
         <is>
           <t>MPA:Dr. Mohd. Prawesh Alam</t>
         </is>
       </c>
-      <c r="E259" s="30" t="inlineStr">
+      <c r="E259" s="27" t="inlineStr">
         <is>
           <t>PSO: PRATEEK KUMAR SONI</t>
         </is>
       </c>
-      <c r="F259" s="30" t="inlineStr">
+      <c r="F259" s="27" t="inlineStr">
         <is>
           <t>SHO: SHOBHIT TYAGI</t>
         </is>
       </c>
-      <c r="G259" s="30" t="inlineStr"/>
-      <c r="H259" s="32" t="inlineStr"/>
-      <c r="I259" s="37" t="inlineStr"/>
+      <c r="G259" s="27" t="inlineStr"/>
+      <c r="H259" s="29" t="inlineStr"/>
+      <c r="I259" s="33" t="inlineStr"/>
       <c r="J259" s="5" t="inlineStr"/>
       <c r="K259" s="1" t="inlineStr"/>
       <c r="L259" s="1" t="inlineStr"/>
@@ -11994,34 +11917,34 @@
     </row>
     <row r="260" ht="15" customHeight="1">
       <c r="A260" s="11" t="n"/>
-      <c r="B260" s="30" t="inlineStr">
+      <c r="B260" s="27" t="inlineStr">
         <is>
           <t>AW: ANKITA</t>
         </is>
       </c>
-      <c r="C260" s="30" t="inlineStr">
+      <c r="C260" s="27" t="inlineStr">
         <is>
           <t>HEM: Hemant Kumar</t>
         </is>
       </c>
-      <c r="D260" s="30" t="inlineStr">
+      <c r="D260" s="27" t="inlineStr">
         <is>
           <t>MSI: MEGH SINGHAL</t>
         </is>
       </c>
-      <c r="E260" s="30" t="inlineStr">
+      <c r="E260" s="27" t="inlineStr">
         <is>
           <t>PTK: PRATIK SHRIVASTAVA</t>
         </is>
       </c>
-      <c r="F260" s="30" t="inlineStr">
+      <c r="F260" s="27" t="inlineStr">
         <is>
           <t>SHR: SHWETA RANI</t>
         </is>
       </c>
-      <c r="G260" s="30" t="inlineStr"/>
-      <c r="H260" s="32" t="inlineStr"/>
-      <c r="I260" s="37" t="inlineStr"/>
+      <c r="G260" s="27" t="inlineStr"/>
+      <c r="H260" s="29" t="inlineStr"/>
+      <c r="I260" s="33" t="inlineStr"/>
       <c r="J260" s="5" t="inlineStr"/>
       <c r="K260" s="1" t="inlineStr"/>
       <c r="L260" s="1" t="inlineStr"/>
@@ -12042,35 +11965,35 @@
     </row>
     <row r="261" ht="15" customHeight="1">
       <c r="A261" s="11" t="n"/>
-      <c r="B261" s="30" t="inlineStr">
+      <c r="B261" s="27" t="inlineStr">
         <is>
           <t>AYS: AYUSH SAHU</t>
         </is>
       </c>
-      <c r="C261" s="30" t="inlineStr">
+      <c r="C261" s="27" t="inlineStr">
         <is>
           <t>HK: HARLEEN KAUR</t>
         </is>
       </c>
-      <c r="D261" s="30" t="inlineStr">
+      <c r="D261" s="27" t="inlineStr">
         <is>
           <t>MTR: Dr. Manoj Tripathi</t>
         </is>
       </c>
-      <c r="E261" s="33" t="inlineStr">
+      <c r="E261" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">RAV: Dr. Ravi Gupta 
 </t>
         </is>
       </c>
-      <c r="F261" s="30" t="inlineStr">
+      <c r="F261" s="27" t="inlineStr">
         <is>
           <t>SHV: SHIVENDRA VIKRAM SINGH</t>
         </is>
       </c>
-      <c r="G261" s="30" t="inlineStr"/>
-      <c r="H261" s="32" t="inlineStr"/>
-      <c r="I261" s="37" t="inlineStr"/>
+      <c r="G261" s="27" t="inlineStr"/>
+      <c r="H261" s="29" t="inlineStr"/>
+      <c r="I261" s="33" t="inlineStr"/>
       <c r="J261" s="5" t="inlineStr"/>
       <c r="K261" s="1" t="inlineStr"/>
       <c r="L261" s="1" t="inlineStr"/>
@@ -12097,8 +12020,8 @@
       <c r="E262" s="12" t="inlineStr"/>
       <c r="F262" s="12" t="inlineStr"/>
       <c r="G262" s="12" t="inlineStr"/>
-      <c r="H262" s="32" t="inlineStr"/>
-      <c r="I262" s="37" t="inlineStr"/>
+      <c r="H262" s="29" t="inlineStr"/>
+      <c r="I262" s="33" t="inlineStr"/>
       <c r="J262" s="5" t="inlineStr"/>
       <c r="K262" s="1" t="inlineStr"/>
       <c r="L262" s="1" t="inlineStr"/>
@@ -12118,13 +12041,13 @@
       <c r="Z262" s="1" t="inlineStr"/>
     </row>
     <row r="263" ht="14.25" customHeight="1">
-      <c r="A263" s="19" t="n"/>
+      <c r="A263" s="17" t="n"/>
       <c r="B263" s="12" t="inlineStr"/>
       <c r="C263" s="12" t="inlineStr"/>
       <c r="D263" s="12" t="inlineStr"/>
       <c r="E263" s="12" t="inlineStr"/>
       <c r="F263" s="12" t="inlineStr"/>
-      <c r="G263" s="33" t="inlineStr"/>
+      <c r="G263" s="30" t="inlineStr"/>
       <c r="H263" s="5" t="inlineStr"/>
       <c r="I263" s="5" t="inlineStr"/>
       <c r="J263" s="5" t="inlineStr"/>

</xml_diff>